<commit_message>
feat(backend): impor Excel menimpa seluruh tabel, tanpa kolom NIK & No. KK
Tanpa NIK tidak ada kunci yang bisa dipercaya untuk mengenali orang yang sama
antar-impor, jadi dedup dihapus bukan diganti: Excel jadi sumber kebenaran
tunggal dan tiap impor mengosongkan tabel lebih dulu. id penduduk kini UUID.
Template & generator data contoh ikut kehilangan dua kolom itu.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/template-data-penduduk.xlsx
+++ b/docs/template-data-penduduk.xlsx
@@ -463,30 +463,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U305"/>
+  <dimension ref="A1:S305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
-    <col width="6" customWidth="1" min="15" max="15"/>
-    <col width="6" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -499,106 +497,96 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>No. KK</t>
+          <t>Nama Lengkap</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>NIK</t>
+          <t>Jenis Kelamin</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Nama Lengkap</t>
+          <t>Tempat Lahir</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Jenis Kelamin</t>
+          <t>Tanggal Lahir (yyyy-mm-dd)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Tempat Lahir</t>
+          <t>Agama</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Tanggal Lahir (yyyy-mm-dd)</t>
+          <t>Status Perkawinan</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Agama</t>
+          <t>Pendidikan Terakhir</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Status Perkawinan</t>
+          <t>Pekerjaan</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Pendidikan Terakhir</t>
+          <t>Gol. Darah</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Pekerjaan</t>
+          <t>Status dalam KK</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Gol. Darah</t>
+          <t>Kewarganegaraan</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Status dalam KK</t>
+          <t>Alamat Jalan</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Kewarganegaraan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Alamat Jalan</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>Desa/Kelurahan</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>Kecamatan</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Desa/Kelurahan</t>
+          <t>Kabupaten</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Kecamatan</t>
+          <t>Provinsi</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>Kabupaten</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>Provinsi</t>
-        </is>
-      </c>
-      <c r="U2" s="2" t="inlineStr">
-        <is>
           <t>Kode Pos</t>
         </is>
       </c>
@@ -606,212 +594,192 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>3204120101900001</t>
+          <t>Contoh Nama Kepala Keluarga</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>3204120101900001</t>
+          <t>LAKI_LAKI</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Contoh Nama Kepala Keluarga</t>
+          <t>Bandung</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>LAKI_LAKI</t>
+          <t>1990-01-01</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Bandung</t>
+          <t>ISLAM</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>1990-01-01</t>
+          <t>KAWIN</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>ISLAM</t>
+          <t>SMA</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>KAWIN</t>
+          <t>Wiraswasta</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>SMA</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Wiraswasta</t>
+          <t>KEPALA_KELUARGA</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>WNI</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>KEPALA_KELUARGA</t>
+          <t>Jl. Contoh No. 1</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>WNI</t>
+          <t>001</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>Jl. Contoh No. 1</t>
+          <t>019</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>Sukamaju</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>019</t>
+          <t>Cibiru</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>Sukamaju</t>
+          <t>Bandung</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>Cibiru</t>
+          <t>Jawa Barat</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
+          <t>40615</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Contoh Nama Istri</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>PEREMPUAN</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t>Bandung</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>1992-05-02</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>ISLAM</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>KAWIN</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Ibu Rumah Tangga</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>ISTRI</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>WNI</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Jl. Contoh No. 1</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>019</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Sukamaju</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Cibiru</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Bandung</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
         </is>
       </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>40615</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>3204120101900001</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>3204124205920002</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Contoh Nama Istri</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>PEREMPUAN</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Bandung</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>1992-05-02</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>ISLAM</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>KAWIN</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>SMA</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Ibu Rumah Tangga</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>ISTRI</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>WNI</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>Jl. Contoh No. 1</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>019</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr">
-        <is>
-          <t>Sukamaju</t>
-        </is>
-      </c>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>Cibiru</t>
-        </is>
-      </c>
       <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>Bandung</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr">
-        <is>
-          <t>Jawa Barat</t>
-        </is>
-      </c>
-      <c r="U4" s="3" t="inlineStr">
         <is>
           <t>40615</t>
         </is>
@@ -837,8 +805,6 @@
       <c r="Q5" s="4" t="n"/>
       <c r="R5" s="4" t="n"/>
       <c r="S5" s="4" t="n"/>
-      <c r="T5" s="4" t="n"/>
-      <c r="U5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n"/>
@@ -860,8 +826,6 @@
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="4" t="n"/>
       <c r="S6" s="4" t="n"/>
-      <c r="T6" s="4" t="n"/>
-      <c r="U6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n"/>
@@ -883,8 +847,6 @@
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="4" t="n"/>
       <c r="S7" s="4" t="n"/>
-      <c r="T7" s="4" t="n"/>
-      <c r="U7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n"/>
@@ -906,8 +868,6 @@
       <c r="Q8" s="4" t="n"/>
       <c r="R8" s="4" t="n"/>
       <c r="S8" s="4" t="n"/>
-      <c r="T8" s="4" t="n"/>
-      <c r="U8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
@@ -929,8 +889,6 @@
       <c r="Q9" s="4" t="n"/>
       <c r="R9" s="4" t="n"/>
       <c r="S9" s="4" t="n"/>
-      <c r="T9" s="4" t="n"/>
-      <c r="U9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
@@ -952,8 +910,6 @@
       <c r="Q10" s="4" t="n"/>
       <c r="R10" s="4" t="n"/>
       <c r="S10" s="4" t="n"/>
-      <c r="T10" s="4" t="n"/>
-      <c r="U10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
@@ -975,8 +931,6 @@
       <c r="Q11" s="4" t="n"/>
       <c r="R11" s="4" t="n"/>
       <c r="S11" s="4" t="n"/>
-      <c r="T11" s="4" t="n"/>
-      <c r="U11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
@@ -998,8 +952,6 @@
       <c r="Q12" s="4" t="n"/>
       <c r="R12" s="4" t="n"/>
       <c r="S12" s="4" t="n"/>
-      <c r="T12" s="4" t="n"/>
-      <c r="U12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
@@ -1021,8 +973,6 @@
       <c r="Q13" s="4" t="n"/>
       <c r="R13" s="4" t="n"/>
       <c r="S13" s="4" t="n"/>
-      <c r="T13" s="4" t="n"/>
-      <c r="U13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
@@ -1044,8 +994,6 @@
       <c r="Q14" s="4" t="n"/>
       <c r="R14" s="4" t="n"/>
       <c r="S14" s="4" t="n"/>
-      <c r="T14" s="4" t="n"/>
-      <c r="U14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
@@ -1067,8 +1015,6 @@
       <c r="Q15" s="4" t="n"/>
       <c r="R15" s="4" t="n"/>
       <c r="S15" s="4" t="n"/>
-      <c r="T15" s="4" t="n"/>
-      <c r="U15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -1090,8 +1036,6 @@
       <c r="Q16" s="4" t="n"/>
       <c r="R16" s="4" t="n"/>
       <c r="S16" s="4" t="n"/>
-      <c r="T16" s="4" t="n"/>
-      <c r="U16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
@@ -1113,8 +1057,6 @@
       <c r="Q17" s="4" t="n"/>
       <c r="R17" s="4" t="n"/>
       <c r="S17" s="4" t="n"/>
-      <c r="T17" s="4" t="n"/>
-      <c r="U17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
@@ -1136,8 +1078,6 @@
       <c r="Q18" s="4" t="n"/>
       <c r="R18" s="4" t="n"/>
       <c r="S18" s="4" t="n"/>
-      <c r="T18" s="4" t="n"/>
-      <c r="U18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
@@ -1159,8 +1099,6 @@
       <c r="Q19" s="4" t="n"/>
       <c r="R19" s="4" t="n"/>
       <c r="S19" s="4" t="n"/>
-      <c r="T19" s="4" t="n"/>
-      <c r="U19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
@@ -1182,8 +1120,6 @@
       <c r="Q20" s="4" t="n"/>
       <c r="R20" s="4" t="n"/>
       <c r="S20" s="4" t="n"/>
-      <c r="T20" s="4" t="n"/>
-      <c r="U20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
@@ -1205,8 +1141,6 @@
       <c r="Q21" s="4" t="n"/>
       <c r="R21" s="4" t="n"/>
       <c r="S21" s="4" t="n"/>
-      <c r="T21" s="4" t="n"/>
-      <c r="U21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>
@@ -1228,8 +1162,6 @@
       <c r="Q22" s="4" t="n"/>
       <c r="R22" s="4" t="n"/>
       <c r="S22" s="4" t="n"/>
-      <c r="T22" s="4" t="n"/>
-      <c r="U22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
@@ -1251,8 +1183,6 @@
       <c r="Q23" s="4" t="n"/>
       <c r="R23" s="4" t="n"/>
       <c r="S23" s="4" t="n"/>
-      <c r="T23" s="4" t="n"/>
-      <c r="U23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n"/>
@@ -1274,8 +1204,6 @@
       <c r="Q24" s="4" t="n"/>
       <c r="R24" s="4" t="n"/>
       <c r="S24" s="4" t="n"/>
-      <c r="T24" s="4" t="n"/>
-      <c r="U24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n"/>
@@ -1297,8 +1225,6 @@
       <c r="Q25" s="4" t="n"/>
       <c r="R25" s="4" t="n"/>
       <c r="S25" s="4" t="n"/>
-      <c r="T25" s="4" t="n"/>
-      <c r="U25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n"/>
@@ -1320,8 +1246,6 @@
       <c r="Q26" s="4" t="n"/>
       <c r="R26" s="4" t="n"/>
       <c r="S26" s="4" t="n"/>
-      <c r="T26" s="4" t="n"/>
-      <c r="U26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n"/>
@@ -1343,8 +1267,6 @@
       <c r="Q27" s="4" t="n"/>
       <c r="R27" s="4" t="n"/>
       <c r="S27" s="4" t="n"/>
-      <c r="T27" s="4" t="n"/>
-      <c r="U27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n"/>
@@ -1366,8 +1288,6 @@
       <c r="Q28" s="4" t="n"/>
       <c r="R28" s="4" t="n"/>
       <c r="S28" s="4" t="n"/>
-      <c r="T28" s="4" t="n"/>
-      <c r="U28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n"/>
@@ -1389,8 +1309,6 @@
       <c r="Q29" s="4" t="n"/>
       <c r="R29" s="4" t="n"/>
       <c r="S29" s="4" t="n"/>
-      <c r="T29" s="4" t="n"/>
-      <c r="U29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n"/>
@@ -1412,8 +1330,6 @@
       <c r="Q30" s="4" t="n"/>
       <c r="R30" s="4" t="n"/>
       <c r="S30" s="4" t="n"/>
-      <c r="T30" s="4" t="n"/>
-      <c r="U30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n"/>
@@ -1435,8 +1351,6 @@
       <c r="Q31" s="4" t="n"/>
       <c r="R31" s="4" t="n"/>
       <c r="S31" s="4" t="n"/>
-      <c r="T31" s="4" t="n"/>
-      <c r="U31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n"/>
@@ -1458,8 +1372,6 @@
       <c r="Q32" s="4" t="n"/>
       <c r="R32" s="4" t="n"/>
       <c r="S32" s="4" t="n"/>
-      <c r="T32" s="4" t="n"/>
-      <c r="U32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
@@ -1481,8 +1393,6 @@
       <c r="Q33" s="4" t="n"/>
       <c r="R33" s="4" t="n"/>
       <c r="S33" s="4" t="n"/>
-      <c r="T33" s="4" t="n"/>
-      <c r="U33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n"/>
@@ -1504,8 +1414,6 @@
       <c r="Q34" s="4" t="n"/>
       <c r="R34" s="4" t="n"/>
       <c r="S34" s="4" t="n"/>
-      <c r="T34" s="4" t="n"/>
-      <c r="U34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n"/>
@@ -1527,8 +1435,6 @@
       <c r="Q35" s="4" t="n"/>
       <c r="R35" s="4" t="n"/>
       <c r="S35" s="4" t="n"/>
-      <c r="T35" s="4" t="n"/>
-      <c r="U35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n"/>
@@ -1550,8 +1456,6 @@
       <c r="Q36" s="4" t="n"/>
       <c r="R36" s="4" t="n"/>
       <c r="S36" s="4" t="n"/>
-      <c r="T36" s="4" t="n"/>
-      <c r="U36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n"/>
@@ -1573,8 +1477,6 @@
       <c r="Q37" s="4" t="n"/>
       <c r="R37" s="4" t="n"/>
       <c r="S37" s="4" t="n"/>
-      <c r="T37" s="4" t="n"/>
-      <c r="U37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n"/>
@@ -1596,8 +1498,6 @@
       <c r="Q38" s="4" t="n"/>
       <c r="R38" s="4" t="n"/>
       <c r="S38" s="4" t="n"/>
-      <c r="T38" s="4" t="n"/>
-      <c r="U38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n"/>
@@ -1619,8 +1519,6 @@
       <c r="Q39" s="4" t="n"/>
       <c r="R39" s="4" t="n"/>
       <c r="S39" s="4" t="n"/>
-      <c r="T39" s="4" t="n"/>
-      <c r="U39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n"/>
@@ -1642,8 +1540,6 @@
       <c r="Q40" s="4" t="n"/>
       <c r="R40" s="4" t="n"/>
       <c r="S40" s="4" t="n"/>
-      <c r="T40" s="4" t="n"/>
-      <c r="U40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n"/>
@@ -1665,8 +1561,6 @@
       <c r="Q41" s="4" t="n"/>
       <c r="R41" s="4" t="n"/>
       <c r="S41" s="4" t="n"/>
-      <c r="T41" s="4" t="n"/>
-      <c r="U41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n"/>
@@ -1688,8 +1582,6 @@
       <c r="Q42" s="4" t="n"/>
       <c r="R42" s="4" t="n"/>
       <c r="S42" s="4" t="n"/>
-      <c r="T42" s="4" t="n"/>
-      <c r="U42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n"/>
@@ -1711,8 +1603,6 @@
       <c r="Q43" s="4" t="n"/>
       <c r="R43" s="4" t="n"/>
       <c r="S43" s="4" t="n"/>
-      <c r="T43" s="4" t="n"/>
-      <c r="U43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n"/>
@@ -1734,8 +1624,6 @@
       <c r="Q44" s="4" t="n"/>
       <c r="R44" s="4" t="n"/>
       <c r="S44" s="4" t="n"/>
-      <c r="T44" s="4" t="n"/>
-      <c r="U44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n"/>
@@ -1757,8 +1645,6 @@
       <c r="Q45" s="4" t="n"/>
       <c r="R45" s="4" t="n"/>
       <c r="S45" s="4" t="n"/>
-      <c r="T45" s="4" t="n"/>
-      <c r="U45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n"/>
@@ -1780,8 +1666,6 @@
       <c r="Q46" s="4" t="n"/>
       <c r="R46" s="4" t="n"/>
       <c r="S46" s="4" t="n"/>
-      <c r="T46" s="4" t="n"/>
-      <c r="U46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n"/>
@@ -1803,8 +1687,6 @@
       <c r="Q47" s="4" t="n"/>
       <c r="R47" s="4" t="n"/>
       <c r="S47" s="4" t="n"/>
-      <c r="T47" s="4" t="n"/>
-      <c r="U47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n"/>
@@ -1826,8 +1708,6 @@
       <c r="Q48" s="4" t="n"/>
       <c r="R48" s="4" t="n"/>
       <c r="S48" s="4" t="n"/>
-      <c r="T48" s="4" t="n"/>
-      <c r="U48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n"/>
@@ -1849,8 +1729,6 @@
       <c r="Q49" s="4" t="n"/>
       <c r="R49" s="4" t="n"/>
       <c r="S49" s="4" t="n"/>
-      <c r="T49" s="4" t="n"/>
-      <c r="U49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n"/>
@@ -1872,8 +1750,6 @@
       <c r="Q50" s="4" t="n"/>
       <c r="R50" s="4" t="n"/>
       <c r="S50" s="4" t="n"/>
-      <c r="T50" s="4" t="n"/>
-      <c r="U50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n"/>
@@ -1895,8 +1771,6 @@
       <c r="Q51" s="4" t="n"/>
       <c r="R51" s="4" t="n"/>
       <c r="S51" s="4" t="n"/>
-      <c r="T51" s="4" t="n"/>
-      <c r="U51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n"/>
@@ -1918,8 +1792,6 @@
       <c r="Q52" s="4" t="n"/>
       <c r="R52" s="4" t="n"/>
       <c r="S52" s="4" t="n"/>
-      <c r="T52" s="4" t="n"/>
-      <c r="U52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n"/>
@@ -1941,8 +1813,6 @@
       <c r="Q53" s="4" t="n"/>
       <c r="R53" s="4" t="n"/>
       <c r="S53" s="4" t="n"/>
-      <c r="T53" s="4" t="n"/>
-      <c r="U53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n"/>
@@ -1964,8 +1834,6 @@
       <c r="Q54" s="4" t="n"/>
       <c r="R54" s="4" t="n"/>
       <c r="S54" s="4" t="n"/>
-      <c r="T54" s="4" t="n"/>
-      <c r="U54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n"/>
@@ -1987,8 +1855,6 @@
       <c r="Q55" s="4" t="n"/>
       <c r="R55" s="4" t="n"/>
       <c r="S55" s="4" t="n"/>
-      <c r="T55" s="4" t="n"/>
-      <c r="U55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n"/>
@@ -2010,8 +1876,6 @@
       <c r="Q56" s="4" t="n"/>
       <c r="R56" s="4" t="n"/>
       <c r="S56" s="4" t="n"/>
-      <c r="T56" s="4" t="n"/>
-      <c r="U56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n"/>
@@ -2033,8 +1897,6 @@
       <c r="Q57" s="4" t="n"/>
       <c r="R57" s="4" t="n"/>
       <c r="S57" s="4" t="n"/>
-      <c r="T57" s="4" t="n"/>
-      <c r="U57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n"/>
@@ -2056,8 +1918,6 @@
       <c r="Q58" s="4" t="n"/>
       <c r="R58" s="4" t="n"/>
       <c r="S58" s="4" t="n"/>
-      <c r="T58" s="4" t="n"/>
-      <c r="U58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n"/>
@@ -2079,8 +1939,6 @@
       <c r="Q59" s="4" t="n"/>
       <c r="R59" s="4" t="n"/>
       <c r="S59" s="4" t="n"/>
-      <c r="T59" s="4" t="n"/>
-      <c r="U59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n"/>
@@ -2102,8 +1960,6 @@
       <c r="Q60" s="4" t="n"/>
       <c r="R60" s="4" t="n"/>
       <c r="S60" s="4" t="n"/>
-      <c r="T60" s="4" t="n"/>
-      <c r="U60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n"/>
@@ -2125,8 +1981,6 @@
       <c r="Q61" s="4" t="n"/>
       <c r="R61" s="4" t="n"/>
       <c r="S61" s="4" t="n"/>
-      <c r="T61" s="4" t="n"/>
-      <c r="U61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n"/>
@@ -2148,8 +2002,6 @@
       <c r="Q62" s="4" t="n"/>
       <c r="R62" s="4" t="n"/>
       <c r="S62" s="4" t="n"/>
-      <c r="T62" s="4" t="n"/>
-      <c r="U62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n"/>
@@ -2171,8 +2023,6 @@
       <c r="Q63" s="4" t="n"/>
       <c r="R63" s="4" t="n"/>
       <c r="S63" s="4" t="n"/>
-      <c r="T63" s="4" t="n"/>
-      <c r="U63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n"/>
@@ -2194,8 +2044,6 @@
       <c r="Q64" s="4" t="n"/>
       <c r="R64" s="4" t="n"/>
       <c r="S64" s="4" t="n"/>
-      <c r="T64" s="4" t="n"/>
-      <c r="U64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n"/>
@@ -2217,8 +2065,6 @@
       <c r="Q65" s="4" t="n"/>
       <c r="R65" s="4" t="n"/>
       <c r="S65" s="4" t="n"/>
-      <c r="T65" s="4" t="n"/>
-      <c r="U65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n"/>
@@ -2240,8 +2086,6 @@
       <c r="Q66" s="4" t="n"/>
       <c r="R66" s="4" t="n"/>
       <c r="S66" s="4" t="n"/>
-      <c r="T66" s="4" t="n"/>
-      <c r="U66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n"/>
@@ -2263,8 +2107,6 @@
       <c r="Q67" s="4" t="n"/>
       <c r="R67" s="4" t="n"/>
       <c r="S67" s="4" t="n"/>
-      <c r="T67" s="4" t="n"/>
-      <c r="U67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="n"/>
@@ -2286,8 +2128,6 @@
       <c r="Q68" s="4" t="n"/>
       <c r="R68" s="4" t="n"/>
       <c r="S68" s="4" t="n"/>
-      <c r="T68" s="4" t="n"/>
-      <c r="U68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n"/>
@@ -2309,8 +2149,6 @@
       <c r="Q69" s="4" t="n"/>
       <c r="R69" s="4" t="n"/>
       <c r="S69" s="4" t="n"/>
-      <c r="T69" s="4" t="n"/>
-      <c r="U69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n"/>
@@ -2332,8 +2170,6 @@
       <c r="Q70" s="4" t="n"/>
       <c r="R70" s="4" t="n"/>
       <c r="S70" s="4" t="n"/>
-      <c r="T70" s="4" t="n"/>
-      <c r="U70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n"/>
@@ -2355,8 +2191,6 @@
       <c r="Q71" s="4" t="n"/>
       <c r="R71" s="4" t="n"/>
       <c r="S71" s="4" t="n"/>
-      <c r="T71" s="4" t="n"/>
-      <c r="U71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n"/>
@@ -2378,8 +2212,6 @@
       <c r="Q72" s="4" t="n"/>
       <c r="R72" s="4" t="n"/>
       <c r="S72" s="4" t="n"/>
-      <c r="T72" s="4" t="n"/>
-      <c r="U72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n"/>
@@ -2401,8 +2233,6 @@
       <c r="Q73" s="4" t="n"/>
       <c r="R73" s="4" t="n"/>
       <c r="S73" s="4" t="n"/>
-      <c r="T73" s="4" t="n"/>
-      <c r="U73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n"/>
@@ -2424,8 +2254,6 @@
       <c r="Q74" s="4" t="n"/>
       <c r="R74" s="4" t="n"/>
       <c r="S74" s="4" t="n"/>
-      <c r="T74" s="4" t="n"/>
-      <c r="U74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n"/>
@@ -2447,8 +2275,6 @@
       <c r="Q75" s="4" t="n"/>
       <c r="R75" s="4" t="n"/>
       <c r="S75" s="4" t="n"/>
-      <c r="T75" s="4" t="n"/>
-      <c r="U75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n"/>
@@ -2470,8 +2296,6 @@
       <c r="Q76" s="4" t="n"/>
       <c r="R76" s="4" t="n"/>
       <c r="S76" s="4" t="n"/>
-      <c r="T76" s="4" t="n"/>
-      <c r="U76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n"/>
@@ -2493,8 +2317,6 @@
       <c r="Q77" s="4" t="n"/>
       <c r="R77" s="4" t="n"/>
       <c r="S77" s="4" t="n"/>
-      <c r="T77" s="4" t="n"/>
-      <c r="U77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n"/>
@@ -2516,8 +2338,6 @@
       <c r="Q78" s="4" t="n"/>
       <c r="R78" s="4" t="n"/>
       <c r="S78" s="4" t="n"/>
-      <c r="T78" s="4" t="n"/>
-      <c r="U78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n"/>
@@ -2539,8 +2359,6 @@
       <c r="Q79" s="4" t="n"/>
       <c r="R79" s="4" t="n"/>
       <c r="S79" s="4" t="n"/>
-      <c r="T79" s="4" t="n"/>
-      <c r="U79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n"/>
@@ -2562,8 +2380,6 @@
       <c r="Q80" s="4" t="n"/>
       <c r="R80" s="4" t="n"/>
       <c r="S80" s="4" t="n"/>
-      <c r="T80" s="4" t="n"/>
-      <c r="U80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n"/>
@@ -2585,8 +2401,6 @@
       <c r="Q81" s="4" t="n"/>
       <c r="R81" s="4" t="n"/>
       <c r="S81" s="4" t="n"/>
-      <c r="T81" s="4" t="n"/>
-      <c r="U81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n"/>
@@ -2608,8 +2422,6 @@
       <c r="Q82" s="4" t="n"/>
       <c r="R82" s="4" t="n"/>
       <c r="S82" s="4" t="n"/>
-      <c r="T82" s="4" t="n"/>
-      <c r="U82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n"/>
@@ -2631,8 +2443,6 @@
       <c r="Q83" s="4" t="n"/>
       <c r="R83" s="4" t="n"/>
       <c r="S83" s="4" t="n"/>
-      <c r="T83" s="4" t="n"/>
-      <c r="U83" s="4" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n"/>
@@ -2654,8 +2464,6 @@
       <c r="Q84" s="4" t="n"/>
       <c r="R84" s="4" t="n"/>
       <c r="S84" s="4" t="n"/>
-      <c r="T84" s="4" t="n"/>
-      <c r="U84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n"/>
@@ -2677,8 +2485,6 @@
       <c r="Q85" s="4" t="n"/>
       <c r="R85" s="4" t="n"/>
       <c r="S85" s="4" t="n"/>
-      <c r="T85" s="4" t="n"/>
-      <c r="U85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="n"/>
@@ -2700,8 +2506,6 @@
       <c r="Q86" s="4" t="n"/>
       <c r="R86" s="4" t="n"/>
       <c r="S86" s="4" t="n"/>
-      <c r="T86" s="4" t="n"/>
-      <c r="U86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n"/>
@@ -2723,8 +2527,6 @@
       <c r="Q87" s="4" t="n"/>
       <c r="R87" s="4" t="n"/>
       <c r="S87" s="4" t="n"/>
-      <c r="T87" s="4" t="n"/>
-      <c r="U87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="n"/>
@@ -2746,8 +2548,6 @@
       <c r="Q88" s="4" t="n"/>
       <c r="R88" s="4" t="n"/>
       <c r="S88" s="4" t="n"/>
-      <c r="T88" s="4" t="n"/>
-      <c r="U88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n"/>
@@ -2769,8 +2569,6 @@
       <c r="Q89" s="4" t="n"/>
       <c r="R89" s="4" t="n"/>
       <c r="S89" s="4" t="n"/>
-      <c r="T89" s="4" t="n"/>
-      <c r="U89" s="4" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n"/>
@@ -2792,8 +2590,6 @@
       <c r="Q90" s="4" t="n"/>
       <c r="R90" s="4" t="n"/>
       <c r="S90" s="4" t="n"/>
-      <c r="T90" s="4" t="n"/>
-      <c r="U90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n"/>
@@ -2815,8 +2611,6 @@
       <c r="Q91" s="4" t="n"/>
       <c r="R91" s="4" t="n"/>
       <c r="S91" s="4" t="n"/>
-      <c r="T91" s="4" t="n"/>
-      <c r="U91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="n"/>
@@ -2838,8 +2632,6 @@
       <c r="Q92" s="4" t="n"/>
       <c r="R92" s="4" t="n"/>
       <c r="S92" s="4" t="n"/>
-      <c r="T92" s="4" t="n"/>
-      <c r="U92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n"/>
@@ -2861,8 +2653,6 @@
       <c r="Q93" s="4" t="n"/>
       <c r="R93" s="4" t="n"/>
       <c r="S93" s="4" t="n"/>
-      <c r="T93" s="4" t="n"/>
-      <c r="U93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="n"/>
@@ -2884,8 +2674,6 @@
       <c r="Q94" s="4" t="n"/>
       <c r="R94" s="4" t="n"/>
       <c r="S94" s="4" t="n"/>
-      <c r="T94" s="4" t="n"/>
-      <c r="U94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n"/>
@@ -2907,8 +2695,6 @@
       <c r="Q95" s="4" t="n"/>
       <c r="R95" s="4" t="n"/>
       <c r="S95" s="4" t="n"/>
-      <c r="T95" s="4" t="n"/>
-      <c r="U95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="n"/>
@@ -2930,8 +2716,6 @@
       <c r="Q96" s="4" t="n"/>
       <c r="R96" s="4" t="n"/>
       <c r="S96" s="4" t="n"/>
-      <c r="T96" s="4" t="n"/>
-      <c r="U96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n"/>
@@ -2953,8 +2737,6 @@
       <c r="Q97" s="4" t="n"/>
       <c r="R97" s="4" t="n"/>
       <c r="S97" s="4" t="n"/>
-      <c r="T97" s="4" t="n"/>
-      <c r="U97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="n"/>
@@ -2976,8 +2758,6 @@
       <c r="Q98" s="4" t="n"/>
       <c r="R98" s="4" t="n"/>
       <c r="S98" s="4" t="n"/>
-      <c r="T98" s="4" t="n"/>
-      <c r="U98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n"/>
@@ -2999,8 +2779,6 @@
       <c r="Q99" s="4" t="n"/>
       <c r="R99" s="4" t="n"/>
       <c r="S99" s="4" t="n"/>
-      <c r="T99" s="4" t="n"/>
-      <c r="U99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="n"/>
@@ -3022,8 +2800,6 @@
       <c r="Q100" s="4" t="n"/>
       <c r="R100" s="4" t="n"/>
       <c r="S100" s="4" t="n"/>
-      <c r="T100" s="4" t="n"/>
-      <c r="U100" s="4" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n"/>
@@ -3045,8 +2821,6 @@
       <c r="Q101" s="4" t="n"/>
       <c r="R101" s="4" t="n"/>
       <c r="S101" s="4" t="n"/>
-      <c r="T101" s="4" t="n"/>
-      <c r="U101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="n"/>
@@ -3068,8 +2842,6 @@
       <c r="Q102" s="4" t="n"/>
       <c r="R102" s="4" t="n"/>
       <c r="S102" s="4" t="n"/>
-      <c r="T102" s="4" t="n"/>
-      <c r="U102" s="4" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="n"/>
@@ -3091,8 +2863,6 @@
       <c r="Q103" s="4" t="n"/>
       <c r="R103" s="4" t="n"/>
       <c r="S103" s="4" t="n"/>
-      <c r="T103" s="4" t="n"/>
-      <c r="U103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="n"/>
@@ -3114,8 +2884,6 @@
       <c r="Q104" s="4" t="n"/>
       <c r="R104" s="4" t="n"/>
       <c r="S104" s="4" t="n"/>
-      <c r="T104" s="4" t="n"/>
-      <c r="U104" s="4" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="n"/>
@@ -3137,8 +2905,6 @@
       <c r="Q105" s="4" t="n"/>
       <c r="R105" s="4" t="n"/>
       <c r="S105" s="4" t="n"/>
-      <c r="T105" s="4" t="n"/>
-      <c r="U105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="n"/>
@@ -3160,8 +2926,6 @@
       <c r="Q106" s="4" t="n"/>
       <c r="R106" s="4" t="n"/>
       <c r="S106" s="4" t="n"/>
-      <c r="T106" s="4" t="n"/>
-      <c r="U106" s="4" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n"/>
@@ -3183,8 +2947,6 @@
       <c r="Q107" s="4" t="n"/>
       <c r="R107" s="4" t="n"/>
       <c r="S107" s="4" t="n"/>
-      <c r="T107" s="4" t="n"/>
-      <c r="U107" s="4" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n"/>
@@ -3206,8 +2968,6 @@
       <c r="Q108" s="4" t="n"/>
       <c r="R108" s="4" t="n"/>
       <c r="S108" s="4" t="n"/>
-      <c r="T108" s="4" t="n"/>
-      <c r="U108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="n"/>
@@ -3229,8 +2989,6 @@
       <c r="Q109" s="4" t="n"/>
       <c r="R109" s="4" t="n"/>
       <c r="S109" s="4" t="n"/>
-      <c r="T109" s="4" t="n"/>
-      <c r="U109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n"/>
@@ -3252,8 +3010,6 @@
       <c r="Q110" s="4" t="n"/>
       <c r="R110" s="4" t="n"/>
       <c r="S110" s="4" t="n"/>
-      <c r="T110" s="4" t="n"/>
-      <c r="U110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n"/>
@@ -3275,8 +3031,6 @@
       <c r="Q111" s="4" t="n"/>
       <c r="R111" s="4" t="n"/>
       <c r="S111" s="4" t="n"/>
-      <c r="T111" s="4" t="n"/>
-      <c r="U111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n"/>
@@ -3298,8 +3052,6 @@
       <c r="Q112" s="4" t="n"/>
       <c r="R112" s="4" t="n"/>
       <c r="S112" s="4" t="n"/>
-      <c r="T112" s="4" t="n"/>
-      <c r="U112" s="4" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n"/>
@@ -3321,8 +3073,6 @@
       <c r="Q113" s="4" t="n"/>
       <c r="R113" s="4" t="n"/>
       <c r="S113" s="4" t="n"/>
-      <c r="T113" s="4" t="n"/>
-      <c r="U113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="n"/>
@@ -3344,8 +3094,6 @@
       <c r="Q114" s="4" t="n"/>
       <c r="R114" s="4" t="n"/>
       <c r="S114" s="4" t="n"/>
-      <c r="T114" s="4" t="n"/>
-      <c r="U114" s="4" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="n"/>
@@ -3367,8 +3115,6 @@
       <c r="Q115" s="4" t="n"/>
       <c r="R115" s="4" t="n"/>
       <c r="S115" s="4" t="n"/>
-      <c r="T115" s="4" t="n"/>
-      <c r="U115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="n"/>
@@ -3390,8 +3136,6 @@
       <c r="Q116" s="4" t="n"/>
       <c r="R116" s="4" t="n"/>
       <c r="S116" s="4" t="n"/>
-      <c r="T116" s="4" t="n"/>
-      <c r="U116" s="4" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n"/>
@@ -3413,8 +3157,6 @@
       <c r="Q117" s="4" t="n"/>
       <c r="R117" s="4" t="n"/>
       <c r="S117" s="4" t="n"/>
-      <c r="T117" s="4" t="n"/>
-      <c r="U117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="n"/>
@@ -3436,8 +3178,6 @@
       <c r="Q118" s="4" t="n"/>
       <c r="R118" s="4" t="n"/>
       <c r="S118" s="4" t="n"/>
-      <c r="T118" s="4" t="n"/>
-      <c r="U118" s="4" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="n"/>
@@ -3459,8 +3199,6 @@
       <c r="Q119" s="4" t="n"/>
       <c r="R119" s="4" t="n"/>
       <c r="S119" s="4" t="n"/>
-      <c r="T119" s="4" t="n"/>
-      <c r="U119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="n"/>
@@ -3482,8 +3220,6 @@
       <c r="Q120" s="4" t="n"/>
       <c r="R120" s="4" t="n"/>
       <c r="S120" s="4" t="n"/>
-      <c r="T120" s="4" t="n"/>
-      <c r="U120" s="4" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="n"/>
@@ -3505,8 +3241,6 @@
       <c r="Q121" s="4" t="n"/>
       <c r="R121" s="4" t="n"/>
       <c r="S121" s="4" t="n"/>
-      <c r="T121" s="4" t="n"/>
-      <c r="U121" s="4" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="n"/>
@@ -3528,8 +3262,6 @@
       <c r="Q122" s="4" t="n"/>
       <c r="R122" s="4" t="n"/>
       <c r="S122" s="4" t="n"/>
-      <c r="T122" s="4" t="n"/>
-      <c r="U122" s="4" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="n"/>
@@ -3551,8 +3283,6 @@
       <c r="Q123" s="4" t="n"/>
       <c r="R123" s="4" t="n"/>
       <c r="S123" s="4" t="n"/>
-      <c r="T123" s="4" t="n"/>
-      <c r="U123" s="4" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="n"/>
@@ -3574,8 +3304,6 @@
       <c r="Q124" s="4" t="n"/>
       <c r="R124" s="4" t="n"/>
       <c r="S124" s="4" t="n"/>
-      <c r="T124" s="4" t="n"/>
-      <c r="U124" s="4" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="n"/>
@@ -3597,8 +3325,6 @@
       <c r="Q125" s="4" t="n"/>
       <c r="R125" s="4" t="n"/>
       <c r="S125" s="4" t="n"/>
-      <c r="T125" s="4" t="n"/>
-      <c r="U125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="n"/>
@@ -3620,8 +3346,6 @@
       <c r="Q126" s="4" t="n"/>
       <c r="R126" s="4" t="n"/>
       <c r="S126" s="4" t="n"/>
-      <c r="T126" s="4" t="n"/>
-      <c r="U126" s="4" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="n"/>
@@ -3643,8 +3367,6 @@
       <c r="Q127" s="4" t="n"/>
       <c r="R127" s="4" t="n"/>
       <c r="S127" s="4" t="n"/>
-      <c r="T127" s="4" t="n"/>
-      <c r="U127" s="4" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="n"/>
@@ -3666,8 +3388,6 @@
       <c r="Q128" s="4" t="n"/>
       <c r="R128" s="4" t="n"/>
       <c r="S128" s="4" t="n"/>
-      <c r="T128" s="4" t="n"/>
-      <c r="U128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="n"/>
@@ -3689,8 +3409,6 @@
       <c r="Q129" s="4" t="n"/>
       <c r="R129" s="4" t="n"/>
       <c r="S129" s="4" t="n"/>
-      <c r="T129" s="4" t="n"/>
-      <c r="U129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="n"/>
@@ -3712,8 +3430,6 @@
       <c r="Q130" s="4" t="n"/>
       <c r="R130" s="4" t="n"/>
       <c r="S130" s="4" t="n"/>
-      <c r="T130" s="4" t="n"/>
-      <c r="U130" s="4" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="n"/>
@@ -3735,8 +3451,6 @@
       <c r="Q131" s="4" t="n"/>
       <c r="R131" s="4" t="n"/>
       <c r="S131" s="4" t="n"/>
-      <c r="T131" s="4" t="n"/>
-      <c r="U131" s="4" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="n"/>
@@ -3758,8 +3472,6 @@
       <c r="Q132" s="4" t="n"/>
       <c r="R132" s="4" t="n"/>
       <c r="S132" s="4" t="n"/>
-      <c r="T132" s="4" t="n"/>
-      <c r="U132" s="4" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="n"/>
@@ -3781,8 +3493,6 @@
       <c r="Q133" s="4" t="n"/>
       <c r="R133" s="4" t="n"/>
       <c r="S133" s="4" t="n"/>
-      <c r="T133" s="4" t="n"/>
-      <c r="U133" s="4" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="n"/>
@@ -3804,8 +3514,6 @@
       <c r="Q134" s="4" t="n"/>
       <c r="R134" s="4" t="n"/>
       <c r="S134" s="4" t="n"/>
-      <c r="T134" s="4" t="n"/>
-      <c r="U134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="n"/>
@@ -3827,8 +3535,6 @@
       <c r="Q135" s="4" t="n"/>
       <c r="R135" s="4" t="n"/>
       <c r="S135" s="4" t="n"/>
-      <c r="T135" s="4" t="n"/>
-      <c r="U135" s="4" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="n"/>
@@ -3850,8 +3556,6 @@
       <c r="Q136" s="4" t="n"/>
       <c r="R136" s="4" t="n"/>
       <c r="S136" s="4" t="n"/>
-      <c r="T136" s="4" t="n"/>
-      <c r="U136" s="4" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n"/>
@@ -3873,8 +3577,6 @@
       <c r="Q137" s="4" t="n"/>
       <c r="R137" s="4" t="n"/>
       <c r="S137" s="4" t="n"/>
-      <c r="T137" s="4" t="n"/>
-      <c r="U137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="n"/>
@@ -3896,8 +3598,6 @@
       <c r="Q138" s="4" t="n"/>
       <c r="R138" s="4" t="n"/>
       <c r="S138" s="4" t="n"/>
-      <c r="T138" s="4" t="n"/>
-      <c r="U138" s="4" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="n"/>
@@ -3919,8 +3619,6 @@
       <c r="Q139" s="4" t="n"/>
       <c r="R139" s="4" t="n"/>
       <c r="S139" s="4" t="n"/>
-      <c r="T139" s="4" t="n"/>
-      <c r="U139" s="4" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="n"/>
@@ -3942,8 +3640,6 @@
       <c r="Q140" s="4" t="n"/>
       <c r="R140" s="4" t="n"/>
       <c r="S140" s="4" t="n"/>
-      <c r="T140" s="4" t="n"/>
-      <c r="U140" s="4" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="n"/>
@@ -3965,8 +3661,6 @@
       <c r="Q141" s="4" t="n"/>
       <c r="R141" s="4" t="n"/>
       <c r="S141" s="4" t="n"/>
-      <c r="T141" s="4" t="n"/>
-      <c r="U141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="n"/>
@@ -3988,8 +3682,6 @@
       <c r="Q142" s="4" t="n"/>
       <c r="R142" s="4" t="n"/>
       <c r="S142" s="4" t="n"/>
-      <c r="T142" s="4" t="n"/>
-      <c r="U142" s="4" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="n"/>
@@ -4011,8 +3703,6 @@
       <c r="Q143" s="4" t="n"/>
       <c r="R143" s="4" t="n"/>
       <c r="S143" s="4" t="n"/>
-      <c r="T143" s="4" t="n"/>
-      <c r="U143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="n"/>
@@ -4034,8 +3724,6 @@
       <c r="Q144" s="4" t="n"/>
       <c r="R144" s="4" t="n"/>
       <c r="S144" s="4" t="n"/>
-      <c r="T144" s="4" t="n"/>
-      <c r="U144" s="4" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="n"/>
@@ -4057,8 +3745,6 @@
       <c r="Q145" s="4" t="n"/>
       <c r="R145" s="4" t="n"/>
       <c r="S145" s="4" t="n"/>
-      <c r="T145" s="4" t="n"/>
-      <c r="U145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="n"/>
@@ -4080,8 +3766,6 @@
       <c r="Q146" s="4" t="n"/>
       <c r="R146" s="4" t="n"/>
       <c r="S146" s="4" t="n"/>
-      <c r="T146" s="4" t="n"/>
-      <c r="U146" s="4" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="n"/>
@@ -4103,8 +3787,6 @@
       <c r="Q147" s="4" t="n"/>
       <c r="R147" s="4" t="n"/>
       <c r="S147" s="4" t="n"/>
-      <c r="T147" s="4" t="n"/>
-      <c r="U147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="n"/>
@@ -4126,8 +3808,6 @@
       <c r="Q148" s="4" t="n"/>
       <c r="R148" s="4" t="n"/>
       <c r="S148" s="4" t="n"/>
-      <c r="T148" s="4" t="n"/>
-      <c r="U148" s="4" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="n"/>
@@ -4149,8 +3829,6 @@
       <c r="Q149" s="4" t="n"/>
       <c r="R149" s="4" t="n"/>
       <c r="S149" s="4" t="n"/>
-      <c r="T149" s="4" t="n"/>
-      <c r="U149" s="4" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="n"/>
@@ -4172,8 +3850,6 @@
       <c r="Q150" s="4" t="n"/>
       <c r="R150" s="4" t="n"/>
       <c r="S150" s="4" t="n"/>
-      <c r="T150" s="4" t="n"/>
-      <c r="U150" s="4" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="n"/>
@@ -4195,8 +3871,6 @@
       <c r="Q151" s="4" t="n"/>
       <c r="R151" s="4" t="n"/>
       <c r="S151" s="4" t="n"/>
-      <c r="T151" s="4" t="n"/>
-      <c r="U151" s="4" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="n"/>
@@ -4218,8 +3892,6 @@
       <c r="Q152" s="4" t="n"/>
       <c r="R152" s="4" t="n"/>
       <c r="S152" s="4" t="n"/>
-      <c r="T152" s="4" t="n"/>
-      <c r="U152" s="4" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="n"/>
@@ -4241,8 +3913,6 @@
       <c r="Q153" s="4" t="n"/>
       <c r="R153" s="4" t="n"/>
       <c r="S153" s="4" t="n"/>
-      <c r="T153" s="4" t="n"/>
-      <c r="U153" s="4" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="n"/>
@@ -4264,8 +3934,6 @@
       <c r="Q154" s="4" t="n"/>
       <c r="R154" s="4" t="n"/>
       <c r="S154" s="4" t="n"/>
-      <c r="T154" s="4" t="n"/>
-      <c r="U154" s="4" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="n"/>
@@ -4287,8 +3955,6 @@
       <c r="Q155" s="4" t="n"/>
       <c r="R155" s="4" t="n"/>
       <c r="S155" s="4" t="n"/>
-      <c r="T155" s="4" t="n"/>
-      <c r="U155" s="4" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="n"/>
@@ -4310,8 +3976,6 @@
       <c r="Q156" s="4" t="n"/>
       <c r="R156" s="4" t="n"/>
       <c r="S156" s="4" t="n"/>
-      <c r="T156" s="4" t="n"/>
-      <c r="U156" s="4" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="n"/>
@@ -4333,8 +3997,6 @@
       <c r="Q157" s="4" t="n"/>
       <c r="R157" s="4" t="n"/>
       <c r="S157" s="4" t="n"/>
-      <c r="T157" s="4" t="n"/>
-      <c r="U157" s="4" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="n"/>
@@ -4356,8 +4018,6 @@
       <c r="Q158" s="4" t="n"/>
       <c r="R158" s="4" t="n"/>
       <c r="S158" s="4" t="n"/>
-      <c r="T158" s="4" t="n"/>
-      <c r="U158" s="4" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n"/>
@@ -4379,8 +4039,6 @@
       <c r="Q159" s="4" t="n"/>
       <c r="R159" s="4" t="n"/>
       <c r="S159" s="4" t="n"/>
-      <c r="T159" s="4" t="n"/>
-      <c r="U159" s="4" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="n"/>
@@ -4402,8 +4060,6 @@
       <c r="Q160" s="4" t="n"/>
       <c r="R160" s="4" t="n"/>
       <c r="S160" s="4" t="n"/>
-      <c r="T160" s="4" t="n"/>
-      <c r="U160" s="4" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="n"/>
@@ -4425,8 +4081,6 @@
       <c r="Q161" s="4" t="n"/>
       <c r="R161" s="4" t="n"/>
       <c r="S161" s="4" t="n"/>
-      <c r="T161" s="4" t="n"/>
-      <c r="U161" s="4" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="n"/>
@@ -4448,8 +4102,6 @@
       <c r="Q162" s="4" t="n"/>
       <c r="R162" s="4" t="n"/>
       <c r="S162" s="4" t="n"/>
-      <c r="T162" s="4" t="n"/>
-      <c r="U162" s="4" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="n"/>
@@ -4471,8 +4123,6 @@
       <c r="Q163" s="4" t="n"/>
       <c r="R163" s="4" t="n"/>
       <c r="S163" s="4" t="n"/>
-      <c r="T163" s="4" t="n"/>
-      <c r="U163" s="4" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="n"/>
@@ -4494,8 +4144,6 @@
       <c r="Q164" s="4" t="n"/>
       <c r="R164" s="4" t="n"/>
       <c r="S164" s="4" t="n"/>
-      <c r="T164" s="4" t="n"/>
-      <c r="U164" s="4" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="n"/>
@@ -4517,8 +4165,6 @@
       <c r="Q165" s="4" t="n"/>
       <c r="R165" s="4" t="n"/>
       <c r="S165" s="4" t="n"/>
-      <c r="T165" s="4" t="n"/>
-      <c r="U165" s="4" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="n"/>
@@ -4540,8 +4186,6 @@
       <c r="Q166" s="4" t="n"/>
       <c r="R166" s="4" t="n"/>
       <c r="S166" s="4" t="n"/>
-      <c r="T166" s="4" t="n"/>
-      <c r="U166" s="4" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="n"/>
@@ -4563,8 +4207,6 @@
       <c r="Q167" s="4" t="n"/>
       <c r="R167" s="4" t="n"/>
       <c r="S167" s="4" t="n"/>
-      <c r="T167" s="4" t="n"/>
-      <c r="U167" s="4" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="n"/>
@@ -4586,8 +4228,6 @@
       <c r="Q168" s="4" t="n"/>
       <c r="R168" s="4" t="n"/>
       <c r="S168" s="4" t="n"/>
-      <c r="T168" s="4" t="n"/>
-      <c r="U168" s="4" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="n"/>
@@ -4609,8 +4249,6 @@
       <c r="Q169" s="4" t="n"/>
       <c r="R169" s="4" t="n"/>
       <c r="S169" s="4" t="n"/>
-      <c r="T169" s="4" t="n"/>
-      <c r="U169" s="4" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="n"/>
@@ -4632,8 +4270,6 @@
       <c r="Q170" s="4" t="n"/>
       <c r="R170" s="4" t="n"/>
       <c r="S170" s="4" t="n"/>
-      <c r="T170" s="4" t="n"/>
-      <c r="U170" s="4" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="n"/>
@@ -4655,8 +4291,6 @@
       <c r="Q171" s="4" t="n"/>
       <c r="R171" s="4" t="n"/>
       <c r="S171" s="4" t="n"/>
-      <c r="T171" s="4" t="n"/>
-      <c r="U171" s="4" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="n"/>
@@ -4678,8 +4312,6 @@
       <c r="Q172" s="4" t="n"/>
       <c r="R172" s="4" t="n"/>
       <c r="S172" s="4" t="n"/>
-      <c r="T172" s="4" t="n"/>
-      <c r="U172" s="4" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="n"/>
@@ -4701,8 +4333,6 @@
       <c r="Q173" s="4" t="n"/>
       <c r="R173" s="4" t="n"/>
       <c r="S173" s="4" t="n"/>
-      <c r="T173" s="4" t="n"/>
-      <c r="U173" s="4" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n"/>
@@ -4724,8 +4354,6 @@
       <c r="Q174" s="4" t="n"/>
       <c r="R174" s="4" t="n"/>
       <c r="S174" s="4" t="n"/>
-      <c r="T174" s="4" t="n"/>
-      <c r="U174" s="4" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="n"/>
@@ -4747,8 +4375,6 @@
       <c r="Q175" s="4" t="n"/>
       <c r="R175" s="4" t="n"/>
       <c r="S175" s="4" t="n"/>
-      <c r="T175" s="4" t="n"/>
-      <c r="U175" s="4" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="n"/>
@@ -4770,8 +4396,6 @@
       <c r="Q176" s="4" t="n"/>
       <c r="R176" s="4" t="n"/>
       <c r="S176" s="4" t="n"/>
-      <c r="T176" s="4" t="n"/>
-      <c r="U176" s="4" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="n"/>
@@ -4793,8 +4417,6 @@
       <c r="Q177" s="4" t="n"/>
       <c r="R177" s="4" t="n"/>
       <c r="S177" s="4" t="n"/>
-      <c r="T177" s="4" t="n"/>
-      <c r="U177" s="4" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="n"/>
@@ -4816,8 +4438,6 @@
       <c r="Q178" s="4" t="n"/>
       <c r="R178" s="4" t="n"/>
       <c r="S178" s="4" t="n"/>
-      <c r="T178" s="4" t="n"/>
-      <c r="U178" s="4" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="n"/>
@@ -4839,8 +4459,6 @@
       <c r="Q179" s="4" t="n"/>
       <c r="R179" s="4" t="n"/>
       <c r="S179" s="4" t="n"/>
-      <c r="T179" s="4" t="n"/>
-      <c r="U179" s="4" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="n"/>
@@ -4862,8 +4480,6 @@
       <c r="Q180" s="4" t="n"/>
       <c r="R180" s="4" t="n"/>
       <c r="S180" s="4" t="n"/>
-      <c r="T180" s="4" t="n"/>
-      <c r="U180" s="4" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="n"/>
@@ -4885,8 +4501,6 @@
       <c r="Q181" s="4" t="n"/>
       <c r="R181" s="4" t="n"/>
       <c r="S181" s="4" t="n"/>
-      <c r="T181" s="4" t="n"/>
-      <c r="U181" s="4" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="n"/>
@@ -4908,8 +4522,6 @@
       <c r="Q182" s="4" t="n"/>
       <c r="R182" s="4" t="n"/>
       <c r="S182" s="4" t="n"/>
-      <c r="T182" s="4" t="n"/>
-      <c r="U182" s="4" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="n"/>
@@ -4931,8 +4543,6 @@
       <c r="Q183" s="4" t="n"/>
       <c r="R183" s="4" t="n"/>
       <c r="S183" s="4" t="n"/>
-      <c r="T183" s="4" t="n"/>
-      <c r="U183" s="4" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="n"/>
@@ -4954,8 +4564,6 @@
       <c r="Q184" s="4" t="n"/>
       <c r="R184" s="4" t="n"/>
       <c r="S184" s="4" t="n"/>
-      <c r="T184" s="4" t="n"/>
-      <c r="U184" s="4" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="n"/>
@@ -4977,8 +4585,6 @@
       <c r="Q185" s="4" t="n"/>
       <c r="R185" s="4" t="n"/>
       <c r="S185" s="4" t="n"/>
-      <c r="T185" s="4" t="n"/>
-      <c r="U185" s="4" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="n"/>
@@ -5000,8 +4606,6 @@
       <c r="Q186" s="4" t="n"/>
       <c r="R186" s="4" t="n"/>
       <c r="S186" s="4" t="n"/>
-      <c r="T186" s="4" t="n"/>
-      <c r="U186" s="4" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="n"/>
@@ -5023,8 +4627,6 @@
       <c r="Q187" s="4" t="n"/>
       <c r="R187" s="4" t="n"/>
       <c r="S187" s="4" t="n"/>
-      <c r="T187" s="4" t="n"/>
-      <c r="U187" s="4" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="n"/>
@@ -5046,8 +4648,6 @@
       <c r="Q188" s="4" t="n"/>
       <c r="R188" s="4" t="n"/>
       <c r="S188" s="4" t="n"/>
-      <c r="T188" s="4" t="n"/>
-      <c r="U188" s="4" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="n"/>
@@ -5069,8 +4669,6 @@
       <c r="Q189" s="4" t="n"/>
       <c r="R189" s="4" t="n"/>
       <c r="S189" s="4" t="n"/>
-      <c r="T189" s="4" t="n"/>
-      <c r="U189" s="4" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="n"/>
@@ -5092,8 +4690,6 @@
       <c r="Q190" s="4" t="n"/>
       <c r="R190" s="4" t="n"/>
       <c r="S190" s="4" t="n"/>
-      <c r="T190" s="4" t="n"/>
-      <c r="U190" s="4" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="n"/>
@@ -5115,8 +4711,6 @@
       <c r="Q191" s="4" t="n"/>
       <c r="R191" s="4" t="n"/>
       <c r="S191" s="4" t="n"/>
-      <c r="T191" s="4" t="n"/>
-      <c r="U191" s="4" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="n"/>
@@ -5138,8 +4732,6 @@
       <c r="Q192" s="4" t="n"/>
       <c r="R192" s="4" t="n"/>
       <c r="S192" s="4" t="n"/>
-      <c r="T192" s="4" t="n"/>
-      <c r="U192" s="4" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="4" t="n"/>
@@ -5161,8 +4753,6 @@
       <c r="Q193" s="4" t="n"/>
       <c r="R193" s="4" t="n"/>
       <c r="S193" s="4" t="n"/>
-      <c r="T193" s="4" t="n"/>
-      <c r="U193" s="4" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="n"/>
@@ -5184,8 +4774,6 @@
       <c r="Q194" s="4" t="n"/>
       <c r="R194" s="4" t="n"/>
       <c r="S194" s="4" t="n"/>
-      <c r="T194" s="4" t="n"/>
-      <c r="U194" s="4" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="n"/>
@@ -5207,8 +4795,6 @@
       <c r="Q195" s="4" t="n"/>
       <c r="R195" s="4" t="n"/>
       <c r="S195" s="4" t="n"/>
-      <c r="T195" s="4" t="n"/>
-      <c r="U195" s="4" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="n"/>
@@ -5230,8 +4816,6 @@
       <c r="Q196" s="4" t="n"/>
       <c r="R196" s="4" t="n"/>
       <c r="S196" s="4" t="n"/>
-      <c r="T196" s="4" t="n"/>
-      <c r="U196" s="4" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="n"/>
@@ -5253,8 +4837,6 @@
       <c r="Q197" s="4" t="n"/>
       <c r="R197" s="4" t="n"/>
       <c r="S197" s="4" t="n"/>
-      <c r="T197" s="4" t="n"/>
-      <c r="U197" s="4" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="n"/>
@@ -5276,8 +4858,6 @@
       <c r="Q198" s="4" t="n"/>
       <c r="R198" s="4" t="n"/>
       <c r="S198" s="4" t="n"/>
-      <c r="T198" s="4" t="n"/>
-      <c r="U198" s="4" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="4" t="n"/>
@@ -5299,8 +4879,6 @@
       <c r="Q199" s="4" t="n"/>
       <c r="R199" s="4" t="n"/>
       <c r="S199" s="4" t="n"/>
-      <c r="T199" s="4" t="n"/>
-      <c r="U199" s="4" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="4" t="n"/>
@@ -5322,8 +4900,6 @@
       <c r="Q200" s="4" t="n"/>
       <c r="R200" s="4" t="n"/>
       <c r="S200" s="4" t="n"/>
-      <c r="T200" s="4" t="n"/>
-      <c r="U200" s="4" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="n"/>
@@ -5345,8 +4921,6 @@
       <c r="Q201" s="4" t="n"/>
       <c r="R201" s="4" t="n"/>
       <c r="S201" s="4" t="n"/>
-      <c r="T201" s="4" t="n"/>
-      <c r="U201" s="4" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="4" t="n"/>
@@ -5368,8 +4942,6 @@
       <c r="Q202" s="4" t="n"/>
       <c r="R202" s="4" t="n"/>
       <c r="S202" s="4" t="n"/>
-      <c r="T202" s="4" t="n"/>
-      <c r="U202" s="4" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="4" t="n"/>
@@ -5391,8 +4963,6 @@
       <c r="Q203" s="4" t="n"/>
       <c r="R203" s="4" t="n"/>
       <c r="S203" s="4" t="n"/>
-      <c r="T203" s="4" t="n"/>
-      <c r="U203" s="4" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="4" t="n"/>
@@ -5414,8 +4984,6 @@
       <c r="Q204" s="4" t="n"/>
       <c r="R204" s="4" t="n"/>
       <c r="S204" s="4" t="n"/>
-      <c r="T204" s="4" t="n"/>
-      <c r="U204" s="4" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="4" t="n"/>
@@ -5437,8 +5005,6 @@
       <c r="Q205" s="4" t="n"/>
       <c r="R205" s="4" t="n"/>
       <c r="S205" s="4" t="n"/>
-      <c r="T205" s="4" t="n"/>
-      <c r="U205" s="4" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="4" t="n"/>
@@ -5460,8 +5026,6 @@
       <c r="Q206" s="4" t="n"/>
       <c r="R206" s="4" t="n"/>
       <c r="S206" s="4" t="n"/>
-      <c r="T206" s="4" t="n"/>
-      <c r="U206" s="4" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="n"/>
@@ -5483,8 +5047,6 @@
       <c r="Q207" s="4" t="n"/>
       <c r="R207" s="4" t="n"/>
       <c r="S207" s="4" t="n"/>
-      <c r="T207" s="4" t="n"/>
-      <c r="U207" s="4" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="4" t="n"/>
@@ -5506,8 +5068,6 @@
       <c r="Q208" s="4" t="n"/>
       <c r="R208" s="4" t="n"/>
       <c r="S208" s="4" t="n"/>
-      <c r="T208" s="4" t="n"/>
-      <c r="U208" s="4" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="4" t="n"/>
@@ -5529,8 +5089,6 @@
       <c r="Q209" s="4" t="n"/>
       <c r="R209" s="4" t="n"/>
       <c r="S209" s="4" t="n"/>
-      <c r="T209" s="4" t="n"/>
-      <c r="U209" s="4" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="n"/>
@@ -5552,8 +5110,6 @@
       <c r="Q210" s="4" t="n"/>
       <c r="R210" s="4" t="n"/>
       <c r="S210" s="4" t="n"/>
-      <c r="T210" s="4" t="n"/>
-      <c r="U210" s="4" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="n"/>
@@ -5575,8 +5131,6 @@
       <c r="Q211" s="4" t="n"/>
       <c r="R211" s="4" t="n"/>
       <c r="S211" s="4" t="n"/>
-      <c r="T211" s="4" t="n"/>
-      <c r="U211" s="4" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="n"/>
@@ -5598,8 +5152,6 @@
       <c r="Q212" s="4" t="n"/>
       <c r="R212" s="4" t="n"/>
       <c r="S212" s="4" t="n"/>
-      <c r="T212" s="4" t="n"/>
-      <c r="U212" s="4" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="4" t="n"/>
@@ -5621,8 +5173,6 @@
       <c r="Q213" s="4" t="n"/>
       <c r="R213" s="4" t="n"/>
       <c r="S213" s="4" t="n"/>
-      <c r="T213" s="4" t="n"/>
-      <c r="U213" s="4" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="n"/>
@@ -5644,8 +5194,6 @@
       <c r="Q214" s="4" t="n"/>
       <c r="R214" s="4" t="n"/>
       <c r="S214" s="4" t="n"/>
-      <c r="T214" s="4" t="n"/>
-      <c r="U214" s="4" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="4" t="n"/>
@@ -5667,8 +5215,6 @@
       <c r="Q215" s="4" t="n"/>
       <c r="R215" s="4" t="n"/>
       <c r="S215" s="4" t="n"/>
-      <c r="T215" s="4" t="n"/>
-      <c r="U215" s="4" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="4" t="n"/>
@@ -5690,8 +5236,6 @@
       <c r="Q216" s="4" t="n"/>
       <c r="R216" s="4" t="n"/>
       <c r="S216" s="4" t="n"/>
-      <c r="T216" s="4" t="n"/>
-      <c r="U216" s="4" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="4" t="n"/>
@@ -5713,8 +5257,6 @@
       <c r="Q217" s="4" t="n"/>
       <c r="R217" s="4" t="n"/>
       <c r="S217" s="4" t="n"/>
-      <c r="T217" s="4" t="n"/>
-      <c r="U217" s="4" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="4" t="n"/>
@@ -5736,8 +5278,6 @@
       <c r="Q218" s="4" t="n"/>
       <c r="R218" s="4" t="n"/>
       <c r="S218" s="4" t="n"/>
-      <c r="T218" s="4" t="n"/>
-      <c r="U218" s="4" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="n"/>
@@ -5759,8 +5299,6 @@
       <c r="Q219" s="4" t="n"/>
       <c r="R219" s="4" t="n"/>
       <c r="S219" s="4" t="n"/>
-      <c r="T219" s="4" t="n"/>
-      <c r="U219" s="4" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="4" t="n"/>
@@ -5782,8 +5320,6 @@
       <c r="Q220" s="4" t="n"/>
       <c r="R220" s="4" t="n"/>
       <c r="S220" s="4" t="n"/>
-      <c r="T220" s="4" t="n"/>
-      <c r="U220" s="4" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="4" t="n"/>
@@ -5805,8 +5341,6 @@
       <c r="Q221" s="4" t="n"/>
       <c r="R221" s="4" t="n"/>
       <c r="S221" s="4" t="n"/>
-      <c r="T221" s="4" t="n"/>
-      <c r="U221" s="4" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="4" t="n"/>
@@ -5828,8 +5362,6 @@
       <c r="Q222" s="4" t="n"/>
       <c r="R222" s="4" t="n"/>
       <c r="S222" s="4" t="n"/>
-      <c r="T222" s="4" t="n"/>
-      <c r="U222" s="4" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="4" t="n"/>
@@ -5851,8 +5383,6 @@
       <c r="Q223" s="4" t="n"/>
       <c r="R223" s="4" t="n"/>
       <c r="S223" s="4" t="n"/>
-      <c r="T223" s="4" t="n"/>
-      <c r="U223" s="4" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="4" t="n"/>
@@ -5874,8 +5404,6 @@
       <c r="Q224" s="4" t="n"/>
       <c r="R224" s="4" t="n"/>
       <c r="S224" s="4" t="n"/>
-      <c r="T224" s="4" t="n"/>
-      <c r="U224" s="4" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="4" t="n"/>
@@ -5897,8 +5425,6 @@
       <c r="Q225" s="4" t="n"/>
       <c r="R225" s="4" t="n"/>
       <c r="S225" s="4" t="n"/>
-      <c r="T225" s="4" t="n"/>
-      <c r="U225" s="4" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="4" t="n"/>
@@ -5920,8 +5446,6 @@
       <c r="Q226" s="4" t="n"/>
       <c r="R226" s="4" t="n"/>
       <c r="S226" s="4" t="n"/>
-      <c r="T226" s="4" t="n"/>
-      <c r="U226" s="4" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="n"/>
@@ -5943,8 +5467,6 @@
       <c r="Q227" s="4" t="n"/>
       <c r="R227" s="4" t="n"/>
       <c r="S227" s="4" t="n"/>
-      <c r="T227" s="4" t="n"/>
-      <c r="U227" s="4" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="4" t="n"/>
@@ -5966,8 +5488,6 @@
       <c r="Q228" s="4" t="n"/>
       <c r="R228" s="4" t="n"/>
       <c r="S228" s="4" t="n"/>
-      <c r="T228" s="4" t="n"/>
-      <c r="U228" s="4" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="4" t="n"/>
@@ -5989,8 +5509,6 @@
       <c r="Q229" s="4" t="n"/>
       <c r="R229" s="4" t="n"/>
       <c r="S229" s="4" t="n"/>
-      <c r="T229" s="4" t="n"/>
-      <c r="U229" s="4" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="4" t="n"/>
@@ -6012,8 +5530,6 @@
       <c r="Q230" s="4" t="n"/>
       <c r="R230" s="4" t="n"/>
       <c r="S230" s="4" t="n"/>
-      <c r="T230" s="4" t="n"/>
-      <c r="U230" s="4" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="n"/>
@@ -6035,8 +5551,6 @@
       <c r="Q231" s="4" t="n"/>
       <c r="R231" s="4" t="n"/>
       <c r="S231" s="4" t="n"/>
-      <c r="T231" s="4" t="n"/>
-      <c r="U231" s="4" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="n"/>
@@ -6058,8 +5572,6 @@
       <c r="Q232" s="4" t="n"/>
       <c r="R232" s="4" t="n"/>
       <c r="S232" s="4" t="n"/>
-      <c r="T232" s="4" t="n"/>
-      <c r="U232" s="4" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="4" t="n"/>
@@ -6081,8 +5593,6 @@
       <c r="Q233" s="4" t="n"/>
       <c r="R233" s="4" t="n"/>
       <c r="S233" s="4" t="n"/>
-      <c r="T233" s="4" t="n"/>
-      <c r="U233" s="4" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="n"/>
@@ -6104,8 +5614,6 @@
       <c r="Q234" s="4" t="n"/>
       <c r="R234" s="4" t="n"/>
       <c r="S234" s="4" t="n"/>
-      <c r="T234" s="4" t="n"/>
-      <c r="U234" s="4" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="4" t="n"/>
@@ -6127,8 +5635,6 @@
       <c r="Q235" s="4" t="n"/>
       <c r="R235" s="4" t="n"/>
       <c r="S235" s="4" t="n"/>
-      <c r="T235" s="4" t="n"/>
-      <c r="U235" s="4" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="4" t="n"/>
@@ -6150,8 +5656,6 @@
       <c r="Q236" s="4" t="n"/>
       <c r="R236" s="4" t="n"/>
       <c r="S236" s="4" t="n"/>
-      <c r="T236" s="4" t="n"/>
-      <c r="U236" s="4" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="4" t="n"/>
@@ -6173,8 +5677,6 @@
       <c r="Q237" s="4" t="n"/>
       <c r="R237" s="4" t="n"/>
       <c r="S237" s="4" t="n"/>
-      <c r="T237" s="4" t="n"/>
-      <c r="U237" s="4" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="4" t="n"/>
@@ -6196,8 +5698,6 @@
       <c r="Q238" s="4" t="n"/>
       <c r="R238" s="4" t="n"/>
       <c r="S238" s="4" t="n"/>
-      <c r="T238" s="4" t="n"/>
-      <c r="U238" s="4" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="4" t="n"/>
@@ -6219,8 +5719,6 @@
       <c r="Q239" s="4" t="n"/>
       <c r="R239" s="4" t="n"/>
       <c r="S239" s="4" t="n"/>
-      <c r="T239" s="4" t="n"/>
-      <c r="U239" s="4" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="4" t="n"/>
@@ -6242,8 +5740,6 @@
       <c r="Q240" s="4" t="n"/>
       <c r="R240" s="4" t="n"/>
       <c r="S240" s="4" t="n"/>
-      <c r="T240" s="4" t="n"/>
-      <c r="U240" s="4" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="4" t="n"/>
@@ -6265,8 +5761,6 @@
       <c r="Q241" s="4" t="n"/>
       <c r="R241" s="4" t="n"/>
       <c r="S241" s="4" t="n"/>
-      <c r="T241" s="4" t="n"/>
-      <c r="U241" s="4" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="4" t="n"/>
@@ -6288,8 +5782,6 @@
       <c r="Q242" s="4" t="n"/>
       <c r="R242" s="4" t="n"/>
       <c r="S242" s="4" t="n"/>
-      <c r="T242" s="4" t="n"/>
-      <c r="U242" s="4" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="4" t="n"/>
@@ -6311,8 +5803,6 @@
       <c r="Q243" s="4" t="n"/>
       <c r="R243" s="4" t="n"/>
       <c r="S243" s="4" t="n"/>
-      <c r="T243" s="4" t="n"/>
-      <c r="U243" s="4" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="n"/>
@@ -6334,8 +5824,6 @@
       <c r="Q244" s="4" t="n"/>
       <c r="R244" s="4" t="n"/>
       <c r="S244" s="4" t="n"/>
-      <c r="T244" s="4" t="n"/>
-      <c r="U244" s="4" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="4" t="n"/>
@@ -6357,8 +5845,6 @@
       <c r="Q245" s="4" t="n"/>
       <c r="R245" s="4" t="n"/>
       <c r="S245" s="4" t="n"/>
-      <c r="T245" s="4" t="n"/>
-      <c r="U245" s="4" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="4" t="n"/>
@@ -6380,8 +5866,6 @@
       <c r="Q246" s="4" t="n"/>
       <c r="R246" s="4" t="n"/>
       <c r="S246" s="4" t="n"/>
-      <c r="T246" s="4" t="n"/>
-      <c r="U246" s="4" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="4" t="n"/>
@@ -6403,8 +5887,6 @@
       <c r="Q247" s="4" t="n"/>
       <c r="R247" s="4" t="n"/>
       <c r="S247" s="4" t="n"/>
-      <c r="T247" s="4" t="n"/>
-      <c r="U247" s="4" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="4" t="n"/>
@@ -6426,8 +5908,6 @@
       <c r="Q248" s="4" t="n"/>
       <c r="R248" s="4" t="n"/>
       <c r="S248" s="4" t="n"/>
-      <c r="T248" s="4" t="n"/>
-      <c r="U248" s="4" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="4" t="n"/>
@@ -6449,8 +5929,6 @@
       <c r="Q249" s="4" t="n"/>
       <c r="R249" s="4" t="n"/>
       <c r="S249" s="4" t="n"/>
-      <c r="T249" s="4" t="n"/>
-      <c r="U249" s="4" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="4" t="n"/>
@@ -6472,8 +5950,6 @@
       <c r="Q250" s="4" t="n"/>
       <c r="R250" s="4" t="n"/>
       <c r="S250" s="4" t="n"/>
-      <c r="T250" s="4" t="n"/>
-      <c r="U250" s="4" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="4" t="n"/>
@@ -6495,8 +5971,6 @@
       <c r="Q251" s="4" t="n"/>
       <c r="R251" s="4" t="n"/>
       <c r="S251" s="4" t="n"/>
-      <c r="T251" s="4" t="n"/>
-      <c r="U251" s="4" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="4" t="n"/>
@@ -6518,8 +5992,6 @@
       <c r="Q252" s="4" t="n"/>
       <c r="R252" s="4" t="n"/>
       <c r="S252" s="4" t="n"/>
-      <c r="T252" s="4" t="n"/>
-      <c r="U252" s="4" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="4" t="n"/>
@@ -6541,8 +6013,6 @@
       <c r="Q253" s="4" t="n"/>
       <c r="R253" s="4" t="n"/>
       <c r="S253" s="4" t="n"/>
-      <c r="T253" s="4" t="n"/>
-      <c r="U253" s="4" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="n"/>
@@ -6564,8 +6034,6 @@
       <c r="Q254" s="4" t="n"/>
       <c r="R254" s="4" t="n"/>
       <c r="S254" s="4" t="n"/>
-      <c r="T254" s="4" t="n"/>
-      <c r="U254" s="4" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="4" t="n"/>
@@ -6587,8 +6055,6 @@
       <c r="Q255" s="4" t="n"/>
       <c r="R255" s="4" t="n"/>
       <c r="S255" s="4" t="n"/>
-      <c r="T255" s="4" t="n"/>
-      <c r="U255" s="4" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="4" t="n"/>
@@ -6610,8 +6076,6 @@
       <c r="Q256" s="4" t="n"/>
       <c r="R256" s="4" t="n"/>
       <c r="S256" s="4" t="n"/>
-      <c r="T256" s="4" t="n"/>
-      <c r="U256" s="4" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="4" t="n"/>
@@ -6633,8 +6097,6 @@
       <c r="Q257" s="4" t="n"/>
       <c r="R257" s="4" t="n"/>
       <c r="S257" s="4" t="n"/>
-      <c r="T257" s="4" t="n"/>
-      <c r="U257" s="4" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="4" t="n"/>
@@ -6656,8 +6118,6 @@
       <c r="Q258" s="4" t="n"/>
       <c r="R258" s="4" t="n"/>
       <c r="S258" s="4" t="n"/>
-      <c r="T258" s="4" t="n"/>
-      <c r="U258" s="4" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="4" t="n"/>
@@ -6679,8 +6139,6 @@
       <c r="Q259" s="4" t="n"/>
       <c r="R259" s="4" t="n"/>
       <c r="S259" s="4" t="n"/>
-      <c r="T259" s="4" t="n"/>
-      <c r="U259" s="4" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="4" t="n"/>
@@ -6702,8 +6160,6 @@
       <c r="Q260" s="4" t="n"/>
       <c r="R260" s="4" t="n"/>
       <c r="S260" s="4" t="n"/>
-      <c r="T260" s="4" t="n"/>
-      <c r="U260" s="4" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="4" t="n"/>
@@ -6725,8 +6181,6 @@
       <c r="Q261" s="4" t="n"/>
       <c r="R261" s="4" t="n"/>
       <c r="S261" s="4" t="n"/>
-      <c r="T261" s="4" t="n"/>
-      <c r="U261" s="4" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="4" t="n"/>
@@ -6748,8 +6202,6 @@
       <c r="Q262" s="4" t="n"/>
       <c r="R262" s="4" t="n"/>
       <c r="S262" s="4" t="n"/>
-      <c r="T262" s="4" t="n"/>
-      <c r="U262" s="4" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="4" t="n"/>
@@ -6771,8 +6223,6 @@
       <c r="Q263" s="4" t="n"/>
       <c r="R263" s="4" t="n"/>
       <c r="S263" s="4" t="n"/>
-      <c r="T263" s="4" t="n"/>
-      <c r="U263" s="4" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="n"/>
@@ -6794,8 +6244,6 @@
       <c r="Q264" s="4" t="n"/>
       <c r="R264" s="4" t="n"/>
       <c r="S264" s="4" t="n"/>
-      <c r="T264" s="4" t="n"/>
-      <c r="U264" s="4" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="4" t="n"/>
@@ -6817,8 +6265,6 @@
       <c r="Q265" s="4" t="n"/>
       <c r="R265" s="4" t="n"/>
       <c r="S265" s="4" t="n"/>
-      <c r="T265" s="4" t="n"/>
-      <c r="U265" s="4" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="n"/>
@@ -6840,8 +6286,6 @@
       <c r="Q266" s="4" t="n"/>
       <c r="R266" s="4" t="n"/>
       <c r="S266" s="4" t="n"/>
-      <c r="T266" s="4" t="n"/>
-      <c r="U266" s="4" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="n"/>
@@ -6863,8 +6307,6 @@
       <c r="Q267" s="4" t="n"/>
       <c r="R267" s="4" t="n"/>
       <c r="S267" s="4" t="n"/>
-      <c r="T267" s="4" t="n"/>
-      <c r="U267" s="4" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="4" t="n"/>
@@ -6886,8 +6328,6 @@
       <c r="Q268" s="4" t="n"/>
       <c r="R268" s="4" t="n"/>
       <c r="S268" s="4" t="n"/>
-      <c r="T268" s="4" t="n"/>
-      <c r="U268" s="4" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="4" t="n"/>
@@ -6909,8 +6349,6 @@
       <c r="Q269" s="4" t="n"/>
       <c r="R269" s="4" t="n"/>
       <c r="S269" s="4" t="n"/>
-      <c r="T269" s="4" t="n"/>
-      <c r="U269" s="4" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="4" t="n"/>
@@ -6932,8 +6370,6 @@
       <c r="Q270" s="4" t="n"/>
       <c r="R270" s="4" t="n"/>
       <c r="S270" s="4" t="n"/>
-      <c r="T270" s="4" t="n"/>
-      <c r="U270" s="4" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="4" t="n"/>
@@ -6955,8 +6391,6 @@
       <c r="Q271" s="4" t="n"/>
       <c r="R271" s="4" t="n"/>
       <c r="S271" s="4" t="n"/>
-      <c r="T271" s="4" t="n"/>
-      <c r="U271" s="4" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="4" t="n"/>
@@ -6978,8 +6412,6 @@
       <c r="Q272" s="4" t="n"/>
       <c r="R272" s="4" t="n"/>
       <c r="S272" s="4" t="n"/>
-      <c r="T272" s="4" t="n"/>
-      <c r="U272" s="4" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="n"/>
@@ -7001,8 +6433,6 @@
       <c r="Q273" s="4" t="n"/>
       <c r="R273" s="4" t="n"/>
       <c r="S273" s="4" t="n"/>
-      <c r="T273" s="4" t="n"/>
-      <c r="U273" s="4" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="4" t="n"/>
@@ -7024,8 +6454,6 @@
       <c r="Q274" s="4" t="n"/>
       <c r="R274" s="4" t="n"/>
       <c r="S274" s="4" t="n"/>
-      <c r="T274" s="4" t="n"/>
-      <c r="U274" s="4" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="4" t="n"/>
@@ -7047,8 +6475,6 @@
       <c r="Q275" s="4" t="n"/>
       <c r="R275" s="4" t="n"/>
       <c r="S275" s="4" t="n"/>
-      <c r="T275" s="4" t="n"/>
-      <c r="U275" s="4" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="n"/>
@@ -7070,8 +6496,6 @@
       <c r="Q276" s="4" t="n"/>
       <c r="R276" s="4" t="n"/>
       <c r="S276" s="4" t="n"/>
-      <c r="T276" s="4" t="n"/>
-      <c r="U276" s="4" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="4" t="n"/>
@@ -7093,8 +6517,6 @@
       <c r="Q277" s="4" t="n"/>
       <c r="R277" s="4" t="n"/>
       <c r="S277" s="4" t="n"/>
-      <c r="T277" s="4" t="n"/>
-      <c r="U277" s="4" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="4" t="n"/>
@@ -7116,8 +6538,6 @@
       <c r="Q278" s="4" t="n"/>
       <c r="R278" s="4" t="n"/>
       <c r="S278" s="4" t="n"/>
-      <c r="T278" s="4" t="n"/>
-      <c r="U278" s="4" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="4" t="n"/>
@@ -7139,8 +6559,6 @@
       <c r="Q279" s="4" t="n"/>
       <c r="R279" s="4" t="n"/>
       <c r="S279" s="4" t="n"/>
-      <c r="T279" s="4" t="n"/>
-      <c r="U279" s="4" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="4" t="n"/>
@@ -7162,8 +6580,6 @@
       <c r="Q280" s="4" t="n"/>
       <c r="R280" s="4" t="n"/>
       <c r="S280" s="4" t="n"/>
-      <c r="T280" s="4" t="n"/>
-      <c r="U280" s="4" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="4" t="n"/>
@@ -7185,8 +6601,6 @@
       <c r="Q281" s="4" t="n"/>
       <c r="R281" s="4" t="n"/>
       <c r="S281" s="4" t="n"/>
-      <c r="T281" s="4" t="n"/>
-      <c r="U281" s="4" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="4" t="n"/>
@@ -7208,8 +6622,6 @@
       <c r="Q282" s="4" t="n"/>
       <c r="R282" s="4" t="n"/>
       <c r="S282" s="4" t="n"/>
-      <c r="T282" s="4" t="n"/>
-      <c r="U282" s="4" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="4" t="n"/>
@@ -7231,8 +6643,6 @@
       <c r="Q283" s="4" t="n"/>
       <c r="R283" s="4" t="n"/>
       <c r="S283" s="4" t="n"/>
-      <c r="T283" s="4" t="n"/>
-      <c r="U283" s="4" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="4" t="n"/>
@@ -7254,8 +6664,6 @@
       <c r="Q284" s="4" t="n"/>
       <c r="R284" s="4" t="n"/>
       <c r="S284" s="4" t="n"/>
-      <c r="T284" s="4" t="n"/>
-      <c r="U284" s="4" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="4" t="n"/>
@@ -7277,8 +6685,6 @@
       <c r="Q285" s="4" t="n"/>
       <c r="R285" s="4" t="n"/>
       <c r="S285" s="4" t="n"/>
-      <c r="T285" s="4" t="n"/>
-      <c r="U285" s="4" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="4" t="n"/>
@@ -7300,8 +6706,6 @@
       <c r="Q286" s="4" t="n"/>
       <c r="R286" s="4" t="n"/>
       <c r="S286" s="4" t="n"/>
-      <c r="T286" s="4" t="n"/>
-      <c r="U286" s="4" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="4" t="n"/>
@@ -7323,8 +6727,6 @@
       <c r="Q287" s="4" t="n"/>
       <c r="R287" s="4" t="n"/>
       <c r="S287" s="4" t="n"/>
-      <c r="T287" s="4" t="n"/>
-      <c r="U287" s="4" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="4" t="n"/>
@@ -7346,8 +6748,6 @@
       <c r="Q288" s="4" t="n"/>
       <c r="R288" s="4" t="n"/>
       <c r="S288" s="4" t="n"/>
-      <c r="T288" s="4" t="n"/>
-      <c r="U288" s="4" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="4" t="n"/>
@@ -7369,8 +6769,6 @@
       <c r="Q289" s="4" t="n"/>
       <c r="R289" s="4" t="n"/>
       <c r="S289" s="4" t="n"/>
-      <c r="T289" s="4" t="n"/>
-      <c r="U289" s="4" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="4" t="n"/>
@@ -7392,8 +6790,6 @@
       <c r="Q290" s="4" t="n"/>
       <c r="R290" s="4" t="n"/>
       <c r="S290" s="4" t="n"/>
-      <c r="T290" s="4" t="n"/>
-      <c r="U290" s="4" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="4" t="n"/>
@@ -7415,8 +6811,6 @@
       <c r="Q291" s="4" t="n"/>
       <c r="R291" s="4" t="n"/>
       <c r="S291" s="4" t="n"/>
-      <c r="T291" s="4" t="n"/>
-      <c r="U291" s="4" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="4" t="n"/>
@@ -7438,8 +6832,6 @@
       <c r="Q292" s="4" t="n"/>
       <c r="R292" s="4" t="n"/>
       <c r="S292" s="4" t="n"/>
-      <c r="T292" s="4" t="n"/>
-      <c r="U292" s="4" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="4" t="n"/>
@@ -7461,8 +6853,6 @@
       <c r="Q293" s="4" t="n"/>
       <c r="R293" s="4" t="n"/>
       <c r="S293" s="4" t="n"/>
-      <c r="T293" s="4" t="n"/>
-      <c r="U293" s="4" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="4" t="n"/>
@@ -7484,8 +6874,6 @@
       <c r="Q294" s="4" t="n"/>
       <c r="R294" s="4" t="n"/>
       <c r="S294" s="4" t="n"/>
-      <c r="T294" s="4" t="n"/>
-      <c r="U294" s="4" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="4" t="n"/>
@@ -7507,8 +6895,6 @@
       <c r="Q295" s="4" t="n"/>
       <c r="R295" s="4" t="n"/>
       <c r="S295" s="4" t="n"/>
-      <c r="T295" s="4" t="n"/>
-      <c r="U295" s="4" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="4" t="n"/>
@@ -7530,8 +6916,6 @@
       <c r="Q296" s="4" t="n"/>
       <c r="R296" s="4" t="n"/>
       <c r="S296" s="4" t="n"/>
-      <c r="T296" s="4" t="n"/>
-      <c r="U296" s="4" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="4" t="n"/>
@@ -7553,8 +6937,6 @@
       <c r="Q297" s="4" t="n"/>
       <c r="R297" s="4" t="n"/>
       <c r="S297" s="4" t="n"/>
-      <c r="T297" s="4" t="n"/>
-      <c r="U297" s="4" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="n"/>
@@ -7576,8 +6958,6 @@
       <c r="Q298" s="4" t="n"/>
       <c r="R298" s="4" t="n"/>
       <c r="S298" s="4" t="n"/>
-      <c r="T298" s="4" t="n"/>
-      <c r="U298" s="4" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="4" t="n"/>
@@ -7599,8 +6979,6 @@
       <c r="Q299" s="4" t="n"/>
       <c r="R299" s="4" t="n"/>
       <c r="S299" s="4" t="n"/>
-      <c r="T299" s="4" t="n"/>
-      <c r="U299" s="4" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n"/>
@@ -7622,8 +7000,6 @@
       <c r="Q300" s="4" t="n"/>
       <c r="R300" s="4" t="n"/>
       <c r="S300" s="4" t="n"/>
-      <c r="T300" s="4" t="n"/>
-      <c r="U300" s="4" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="4" t="n"/>
@@ -7645,8 +7021,6 @@
       <c r="Q301" s="4" t="n"/>
       <c r="R301" s="4" t="n"/>
       <c r="S301" s="4" t="n"/>
-      <c r="T301" s="4" t="n"/>
-      <c r="U301" s="4" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="4" t="n"/>
@@ -7668,8 +7042,6 @@
       <c r="Q302" s="4" t="n"/>
       <c r="R302" s="4" t="n"/>
       <c r="S302" s="4" t="n"/>
-      <c r="T302" s="4" t="n"/>
-      <c r="U302" s="4" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="n"/>
@@ -7691,8 +7063,6 @@
       <c r="Q303" s="4" t="n"/>
       <c r="R303" s="4" t="n"/>
       <c r="S303" s="4" t="n"/>
-      <c r="T303" s="4" t="n"/>
-      <c r="U303" s="4" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="4" t="n"/>
@@ -7714,8 +7084,6 @@
       <c r="Q304" s="4" t="n"/>
       <c r="R304" s="4" t="n"/>
       <c r="S304" s="4" t="n"/>
-      <c r="T304" s="4" t="n"/>
-      <c r="U304" s="4" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="4" t="n"/>
@@ -7737,30 +7105,28 @@
       <c r="Q305" s="4" t="n"/>
       <c r="R305" s="4" t="n"/>
       <c r="S305" s="4" t="n"/>
-      <c r="T305" s="4" t="n"/>
-      <c r="U305" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A1:S1"/>
   </mergeCells>
   <dataValidations count="6">
-    <dataValidation sqref="D3:D305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: LAKI_LAKI, PEREMPUAN" type="list">
+    <dataValidation sqref="B3:B305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: LAKI_LAKI, PEREMPUAN" type="list">
       <formula1>"LAKI_LAKI,PEREMPUAN"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: ISLAM, KRISTEN, KATOLIK, HINDU, BUDDHA, KONGHUCU, LAINNYA" type="list">
+    <dataValidation sqref="E3:E305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: ISLAM, KRISTEN, KATOLIK, HINDU, BUDDHA, KONGHUCU, LAINNYA" type="list">
       <formula1>"ISLAM,KRISTEN,KATOLIK,HINDU,BUDDHA,KONGHUCU,LAINNYA"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: BELUM_KAWIN, KAWIN, CERAI_HIDUP, CERAI_MATI" type="list">
+    <dataValidation sqref="F3:F305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: BELUM_KAWIN, KAWIN, CERAI_HIDUP, CERAI_MATI" type="list">
       <formula1>"BELUM_KAWIN,KAWIN,CERAI_HIDUP,CERAI_MATI"</formula1>
     </dataValidation>
-    <dataValidation sqref="I3:I305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: TIDAK_SEKOLAH, SD, SMP, SMA, D3, S1, S2, S3" type="list">
+    <dataValidation sqref="G3:G305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: TIDAK_SEKOLAH, SD, SMP, SMA, D3, S1, S2, S3" type="list">
       <formula1>"TIDAK_SEKOLAH,SD,SMP,SMA,D3,S1,S2,S3"</formula1>
     </dataValidation>
-    <dataValidation sqref="K3:K305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: A, B, AB, O, TIDAK_TAHU" type="list">
+    <dataValidation sqref="I3:I305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: A, B, AB, O, TIDAK_TAHU" type="list">
       <formula1>"A,B,AB,O,TIDAK_TAHU"</formula1>
     </dataValidation>
-    <dataValidation sqref="L3:L305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: KEPALA_KELUARGA, ISTRI, ANAK, FAMILI_LAIN, LAINNYA" type="list">
+    <dataValidation sqref="J3:J305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: KEPALA_KELUARGA, ISTRI, ANAK, FAMILI_LAIN, LAINNYA" type="list">
       <formula1>"KEPALA_KELUARGA,ISTRI,ANAK,FAMILI_LAIN,LAINNYA"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7774,7 +7140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -7807,28 +7173,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. NIK dan No. KK: 16 digit angka, tanpa spasi atau tanda baca.</t>
+          <t>3. NIK dan No. KK TIDAK didata. Jangan menambahkan kolomnya sendiri —</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4. Satu keluarga = satu No. KK yang sama di semua anggotanya.</t>
+          <t xml:space="preserve">   sistem tidak menyimpannya, dan desa tidak mengizinkannya.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5. Tanggal Lahir: format yyyy-mm-dd (contoh 1990-01-01).</t>
+          <t>4. Tanggal Lahir: format yyyy-mm-dd (contoh 1990-01-01).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6. Kolom berikut WAJIB pilih dari dropdown (klik sel, muncul panah di kanan):</t>
+          <t>5. Kolom berikut WAJIB pilih dari dropdown (klik sel, muncul panah di kanan):</t>
         </is>
       </c>
     </row>
@@ -7842,12 +7208,26 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Gol. Darah, Status dalam KK.</t>
+          <t xml:space="preserve">   Gol. Darah, Status dalam Keluarga.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>6. Kirim file LENGKAP berisi SELURUH warga, bukan tambahannya saja:</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   impor menimpa seluruh data lama.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>7. Simpan sebagai .xlsx, kirim ke pengelola data untuk diimpor ke sistem.</t>
         </is>

</xml_diff>

<commit_message>
feat(backend): empat peran, kursi pengurus, dan Kode Warga sebagai id warga
ADMIN/DUKUH/RW/RT. ADMIN kehilangan seluruh akses data warga (current_pengurus
menolaknya); DUKUH/RW/RT tidak bisa menyentuh akun. GET /pengurus sekarang
mengembalikan kursi — diturunkan dari alamat warga, terisi maupun kosong —
bukan sekadar daftar akun, dan satu kursi hanya boleh dihuni satu akun aktif.

Kolom Kode Warga di Excel menjadi id penduduk menggantikan UUID: jabatan
pengurus harus bisa menunjuk warga tertentu, sementara impor menimpa seluruh
tabel. Kode ganda atau kosong menghentikan impor sebelum satu baris ditulis.

Password awal dari Admin sekali pakai: akun baru bisa login tapi ditolak di
semua endpoint lain sampai menggantinya sendiri lewat POST /auth/ganti-password.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/template-data-penduduk.xlsx
+++ b/docs/template-data-penduduk.xlsx
@@ -463,28 +463,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S305"/>
+  <dimension ref="A1:T305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
     <col width="6" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -497,95 +498,100 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Kode Warga</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>Nama Lengkap</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Jenis Kelamin</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Tempat Lahir</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Tanggal Lahir (yyyy-mm-dd)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Agama</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Status Perkawinan</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Pendidikan Terakhir</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Pekerjaan</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Gol. Darah</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Status dalam KK</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Kewarganegaraan</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Alamat Jalan</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>RT</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>RW</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Desa/Kelurahan</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Kecamatan</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Kabupaten</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Provinsi</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Kode Pos</t>
         </is>
@@ -594,95 +600,100 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
+          <t>W0001</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
           <t>Contoh Nama Kepala Keluarga</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>LAKI_LAKI</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Bandung</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>1990-01-01</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>ISLAM</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>KAWIN</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>SMA</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Wiraswasta</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>KEPALA_KELUARGA</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>WNI</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Jl. Contoh No. 1</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>019</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Sukamaju</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>Cibiru</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>Bandung</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>40615</t>
         </is>
@@ -691,95 +702,100 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
+          <t>W0002</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
           <t>Contoh Nama Istri</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>PEREMPUAN</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Bandung</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>1992-05-02</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>ISLAM</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>KAWIN</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>SMA</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Ibu Rumah Tangga</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>ISTRI</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>WNI</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Jl. Contoh No. 1</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>019</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Sukamaju</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Cibiru</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Bandung</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>40615</t>
         </is>
@@ -805,6 +821,7 @@
       <c r="Q5" s="4" t="n"/>
       <c r="R5" s="4" t="n"/>
       <c r="S5" s="4" t="n"/>
+      <c r="T5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n"/>
@@ -826,6 +843,7 @@
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="4" t="n"/>
       <c r="S6" s="4" t="n"/>
+      <c r="T6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n"/>
@@ -847,6 +865,7 @@
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="4" t="n"/>
       <c r="S7" s="4" t="n"/>
+      <c r="T7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n"/>
@@ -868,6 +887,7 @@
       <c r="Q8" s="4" t="n"/>
       <c r="R8" s="4" t="n"/>
       <c r="S8" s="4" t="n"/>
+      <c r="T8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
@@ -889,6 +909,7 @@
       <c r="Q9" s="4" t="n"/>
       <c r="R9" s="4" t="n"/>
       <c r="S9" s="4" t="n"/>
+      <c r="T9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
@@ -910,6 +931,7 @@
       <c r="Q10" s="4" t="n"/>
       <c r="R10" s="4" t="n"/>
       <c r="S10" s="4" t="n"/>
+      <c r="T10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
@@ -931,6 +953,7 @@
       <c r="Q11" s="4" t="n"/>
       <c r="R11" s="4" t="n"/>
       <c r="S11" s="4" t="n"/>
+      <c r="T11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
@@ -952,6 +975,7 @@
       <c r="Q12" s="4" t="n"/>
       <c r="R12" s="4" t="n"/>
       <c r="S12" s="4" t="n"/>
+      <c r="T12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
@@ -973,6 +997,7 @@
       <c r="Q13" s="4" t="n"/>
       <c r="R13" s="4" t="n"/>
       <c r="S13" s="4" t="n"/>
+      <c r="T13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
@@ -994,6 +1019,7 @@
       <c r="Q14" s="4" t="n"/>
       <c r="R14" s="4" t="n"/>
       <c r="S14" s="4" t="n"/>
+      <c r="T14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
@@ -1015,6 +1041,7 @@
       <c r="Q15" s="4" t="n"/>
       <c r="R15" s="4" t="n"/>
       <c r="S15" s="4" t="n"/>
+      <c r="T15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -1036,6 +1063,7 @@
       <c r="Q16" s="4" t="n"/>
       <c r="R16" s="4" t="n"/>
       <c r="S16" s="4" t="n"/>
+      <c r="T16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
@@ -1057,6 +1085,7 @@
       <c r="Q17" s="4" t="n"/>
       <c r="R17" s="4" t="n"/>
       <c r="S17" s="4" t="n"/>
+      <c r="T17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
@@ -1078,6 +1107,7 @@
       <c r="Q18" s="4" t="n"/>
       <c r="R18" s="4" t="n"/>
       <c r="S18" s="4" t="n"/>
+      <c r="T18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
@@ -1099,6 +1129,7 @@
       <c r="Q19" s="4" t="n"/>
       <c r="R19" s="4" t="n"/>
       <c r="S19" s="4" t="n"/>
+      <c r="T19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
@@ -1120,6 +1151,7 @@
       <c r="Q20" s="4" t="n"/>
       <c r="R20" s="4" t="n"/>
       <c r="S20" s="4" t="n"/>
+      <c r="T20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
@@ -1141,6 +1173,7 @@
       <c r="Q21" s="4" t="n"/>
       <c r="R21" s="4" t="n"/>
       <c r="S21" s="4" t="n"/>
+      <c r="T21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>
@@ -1162,6 +1195,7 @@
       <c r="Q22" s="4" t="n"/>
       <c r="R22" s="4" t="n"/>
       <c r="S22" s="4" t="n"/>
+      <c r="T22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
@@ -1183,6 +1217,7 @@
       <c r="Q23" s="4" t="n"/>
       <c r="R23" s="4" t="n"/>
       <c r="S23" s="4" t="n"/>
+      <c r="T23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n"/>
@@ -1204,6 +1239,7 @@
       <c r="Q24" s="4" t="n"/>
       <c r="R24" s="4" t="n"/>
       <c r="S24" s="4" t="n"/>
+      <c r="T24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n"/>
@@ -1225,6 +1261,7 @@
       <c r="Q25" s="4" t="n"/>
       <c r="R25" s="4" t="n"/>
       <c r="S25" s="4" t="n"/>
+      <c r="T25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n"/>
@@ -1246,6 +1283,7 @@
       <c r="Q26" s="4" t="n"/>
       <c r="R26" s="4" t="n"/>
       <c r="S26" s="4" t="n"/>
+      <c r="T26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n"/>
@@ -1267,6 +1305,7 @@
       <c r="Q27" s="4" t="n"/>
       <c r="R27" s="4" t="n"/>
       <c r="S27" s="4" t="n"/>
+      <c r="T27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n"/>
@@ -1288,6 +1327,7 @@
       <c r="Q28" s="4" t="n"/>
       <c r="R28" s="4" t="n"/>
       <c r="S28" s="4" t="n"/>
+      <c r="T28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n"/>
@@ -1309,6 +1349,7 @@
       <c r="Q29" s="4" t="n"/>
       <c r="R29" s="4" t="n"/>
       <c r="S29" s="4" t="n"/>
+      <c r="T29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n"/>
@@ -1330,6 +1371,7 @@
       <c r="Q30" s="4" t="n"/>
       <c r="R30" s="4" t="n"/>
       <c r="S30" s="4" t="n"/>
+      <c r="T30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n"/>
@@ -1351,6 +1393,7 @@
       <c r="Q31" s="4" t="n"/>
       <c r="R31" s="4" t="n"/>
       <c r="S31" s="4" t="n"/>
+      <c r="T31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n"/>
@@ -1372,6 +1415,7 @@
       <c r="Q32" s="4" t="n"/>
       <c r="R32" s="4" t="n"/>
       <c r="S32" s="4" t="n"/>
+      <c r="T32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
@@ -1393,6 +1437,7 @@
       <c r="Q33" s="4" t="n"/>
       <c r="R33" s="4" t="n"/>
       <c r="S33" s="4" t="n"/>
+      <c r="T33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n"/>
@@ -1414,6 +1459,7 @@
       <c r="Q34" s="4" t="n"/>
       <c r="R34" s="4" t="n"/>
       <c r="S34" s="4" t="n"/>
+      <c r="T34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n"/>
@@ -1435,6 +1481,7 @@
       <c r="Q35" s="4" t="n"/>
       <c r="R35" s="4" t="n"/>
       <c r="S35" s="4" t="n"/>
+      <c r="T35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n"/>
@@ -1456,6 +1503,7 @@
       <c r="Q36" s="4" t="n"/>
       <c r="R36" s="4" t="n"/>
       <c r="S36" s="4" t="n"/>
+      <c r="T36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n"/>
@@ -1477,6 +1525,7 @@
       <c r="Q37" s="4" t="n"/>
       <c r="R37" s="4" t="n"/>
       <c r="S37" s="4" t="n"/>
+      <c r="T37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n"/>
@@ -1498,6 +1547,7 @@
       <c r="Q38" s="4" t="n"/>
       <c r="R38" s="4" t="n"/>
       <c r="S38" s="4" t="n"/>
+      <c r="T38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n"/>
@@ -1519,6 +1569,7 @@
       <c r="Q39" s="4" t="n"/>
       <c r="R39" s="4" t="n"/>
       <c r="S39" s="4" t="n"/>
+      <c r="T39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n"/>
@@ -1540,6 +1591,7 @@
       <c r="Q40" s="4" t="n"/>
       <c r="R40" s="4" t="n"/>
       <c r="S40" s="4" t="n"/>
+      <c r="T40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n"/>
@@ -1561,6 +1613,7 @@
       <c r="Q41" s="4" t="n"/>
       <c r="R41" s="4" t="n"/>
       <c r="S41" s="4" t="n"/>
+      <c r="T41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n"/>
@@ -1582,6 +1635,7 @@
       <c r="Q42" s="4" t="n"/>
       <c r="R42" s="4" t="n"/>
       <c r="S42" s="4" t="n"/>
+      <c r="T42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n"/>
@@ -1603,6 +1657,7 @@
       <c r="Q43" s="4" t="n"/>
       <c r="R43" s="4" t="n"/>
       <c r="S43" s="4" t="n"/>
+      <c r="T43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n"/>
@@ -1624,6 +1679,7 @@
       <c r="Q44" s="4" t="n"/>
       <c r="R44" s="4" t="n"/>
       <c r="S44" s="4" t="n"/>
+      <c r="T44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n"/>
@@ -1645,6 +1701,7 @@
       <c r="Q45" s="4" t="n"/>
       <c r="R45" s="4" t="n"/>
       <c r="S45" s="4" t="n"/>
+      <c r="T45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n"/>
@@ -1666,6 +1723,7 @@
       <c r="Q46" s="4" t="n"/>
       <c r="R46" s="4" t="n"/>
       <c r="S46" s="4" t="n"/>
+      <c r="T46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n"/>
@@ -1687,6 +1745,7 @@
       <c r="Q47" s="4" t="n"/>
       <c r="R47" s="4" t="n"/>
       <c r="S47" s="4" t="n"/>
+      <c r="T47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n"/>
@@ -1708,6 +1767,7 @@
       <c r="Q48" s="4" t="n"/>
       <c r="R48" s="4" t="n"/>
       <c r="S48" s="4" t="n"/>
+      <c r="T48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n"/>
@@ -1729,6 +1789,7 @@
       <c r="Q49" s="4" t="n"/>
       <c r="R49" s="4" t="n"/>
       <c r="S49" s="4" t="n"/>
+      <c r="T49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n"/>
@@ -1750,6 +1811,7 @@
       <c r="Q50" s="4" t="n"/>
       <c r="R50" s="4" t="n"/>
       <c r="S50" s="4" t="n"/>
+      <c r="T50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n"/>
@@ -1771,6 +1833,7 @@
       <c r="Q51" s="4" t="n"/>
       <c r="R51" s="4" t="n"/>
       <c r="S51" s="4" t="n"/>
+      <c r="T51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n"/>
@@ -1792,6 +1855,7 @@
       <c r="Q52" s="4" t="n"/>
       <c r="R52" s="4" t="n"/>
       <c r="S52" s="4" t="n"/>
+      <c r="T52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n"/>
@@ -1813,6 +1877,7 @@
       <c r="Q53" s="4" t="n"/>
       <c r="R53" s="4" t="n"/>
       <c r="S53" s="4" t="n"/>
+      <c r="T53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n"/>
@@ -1834,6 +1899,7 @@
       <c r="Q54" s="4" t="n"/>
       <c r="R54" s="4" t="n"/>
       <c r="S54" s="4" t="n"/>
+      <c r="T54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n"/>
@@ -1855,6 +1921,7 @@
       <c r="Q55" s="4" t="n"/>
       <c r="R55" s="4" t="n"/>
       <c r="S55" s="4" t="n"/>
+      <c r="T55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n"/>
@@ -1876,6 +1943,7 @@
       <c r="Q56" s="4" t="n"/>
       <c r="R56" s="4" t="n"/>
       <c r="S56" s="4" t="n"/>
+      <c r="T56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n"/>
@@ -1897,6 +1965,7 @@
       <c r="Q57" s="4" t="n"/>
       <c r="R57" s="4" t="n"/>
       <c r="S57" s="4" t="n"/>
+      <c r="T57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n"/>
@@ -1918,6 +1987,7 @@
       <c r="Q58" s="4" t="n"/>
       <c r="R58" s="4" t="n"/>
       <c r="S58" s="4" t="n"/>
+      <c r="T58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n"/>
@@ -1939,6 +2009,7 @@
       <c r="Q59" s="4" t="n"/>
       <c r="R59" s="4" t="n"/>
       <c r="S59" s="4" t="n"/>
+      <c r="T59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n"/>
@@ -1960,6 +2031,7 @@
       <c r="Q60" s="4" t="n"/>
       <c r="R60" s="4" t="n"/>
       <c r="S60" s="4" t="n"/>
+      <c r="T60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n"/>
@@ -1981,6 +2053,7 @@
       <c r="Q61" s="4" t="n"/>
       <c r="R61" s="4" t="n"/>
       <c r="S61" s="4" t="n"/>
+      <c r="T61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n"/>
@@ -2002,6 +2075,7 @@
       <c r="Q62" s="4" t="n"/>
       <c r="R62" s="4" t="n"/>
       <c r="S62" s="4" t="n"/>
+      <c r="T62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n"/>
@@ -2023,6 +2097,7 @@
       <c r="Q63" s="4" t="n"/>
       <c r="R63" s="4" t="n"/>
       <c r="S63" s="4" t="n"/>
+      <c r="T63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n"/>
@@ -2044,6 +2119,7 @@
       <c r="Q64" s="4" t="n"/>
       <c r="R64" s="4" t="n"/>
       <c r="S64" s="4" t="n"/>
+      <c r="T64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n"/>
@@ -2065,6 +2141,7 @@
       <c r="Q65" s="4" t="n"/>
       <c r="R65" s="4" t="n"/>
       <c r="S65" s="4" t="n"/>
+      <c r="T65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n"/>
@@ -2086,6 +2163,7 @@
       <c r="Q66" s="4" t="n"/>
       <c r="R66" s="4" t="n"/>
       <c r="S66" s="4" t="n"/>
+      <c r="T66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n"/>
@@ -2107,6 +2185,7 @@
       <c r="Q67" s="4" t="n"/>
       <c r="R67" s="4" t="n"/>
       <c r="S67" s="4" t="n"/>
+      <c r="T67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="n"/>
@@ -2128,6 +2207,7 @@
       <c r="Q68" s="4" t="n"/>
       <c r="R68" s="4" t="n"/>
       <c r="S68" s="4" t="n"/>
+      <c r="T68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n"/>
@@ -2149,6 +2229,7 @@
       <c r="Q69" s="4" t="n"/>
       <c r="R69" s="4" t="n"/>
       <c r="S69" s="4" t="n"/>
+      <c r="T69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n"/>
@@ -2170,6 +2251,7 @@
       <c r="Q70" s="4" t="n"/>
       <c r="R70" s="4" t="n"/>
       <c r="S70" s="4" t="n"/>
+      <c r="T70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n"/>
@@ -2191,6 +2273,7 @@
       <c r="Q71" s="4" t="n"/>
       <c r="R71" s="4" t="n"/>
       <c r="S71" s="4" t="n"/>
+      <c r="T71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n"/>
@@ -2212,6 +2295,7 @@
       <c r="Q72" s="4" t="n"/>
       <c r="R72" s="4" t="n"/>
       <c r="S72" s="4" t="n"/>
+      <c r="T72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n"/>
@@ -2233,6 +2317,7 @@
       <c r="Q73" s="4" t="n"/>
       <c r="R73" s="4" t="n"/>
       <c r="S73" s="4" t="n"/>
+      <c r="T73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n"/>
@@ -2254,6 +2339,7 @@
       <c r="Q74" s="4" t="n"/>
       <c r="R74" s="4" t="n"/>
       <c r="S74" s="4" t="n"/>
+      <c r="T74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n"/>
@@ -2275,6 +2361,7 @@
       <c r="Q75" s="4" t="n"/>
       <c r="R75" s="4" t="n"/>
       <c r="S75" s="4" t="n"/>
+      <c r="T75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n"/>
@@ -2296,6 +2383,7 @@
       <c r="Q76" s="4" t="n"/>
       <c r="R76" s="4" t="n"/>
       <c r="S76" s="4" t="n"/>
+      <c r="T76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n"/>
@@ -2317,6 +2405,7 @@
       <c r="Q77" s="4" t="n"/>
       <c r="R77" s="4" t="n"/>
       <c r="S77" s="4" t="n"/>
+      <c r="T77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n"/>
@@ -2338,6 +2427,7 @@
       <c r="Q78" s="4" t="n"/>
       <c r="R78" s="4" t="n"/>
       <c r="S78" s="4" t="n"/>
+      <c r="T78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n"/>
@@ -2359,6 +2449,7 @@
       <c r="Q79" s="4" t="n"/>
       <c r="R79" s="4" t="n"/>
       <c r="S79" s="4" t="n"/>
+      <c r="T79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n"/>
@@ -2380,6 +2471,7 @@
       <c r="Q80" s="4" t="n"/>
       <c r="R80" s="4" t="n"/>
       <c r="S80" s="4" t="n"/>
+      <c r="T80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n"/>
@@ -2401,6 +2493,7 @@
       <c r="Q81" s="4" t="n"/>
       <c r="R81" s="4" t="n"/>
       <c r="S81" s="4" t="n"/>
+      <c r="T81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n"/>
@@ -2422,6 +2515,7 @@
       <c r="Q82" s="4" t="n"/>
       <c r="R82" s="4" t="n"/>
       <c r="S82" s="4" t="n"/>
+      <c r="T82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n"/>
@@ -2443,6 +2537,7 @@
       <c r="Q83" s="4" t="n"/>
       <c r="R83" s="4" t="n"/>
       <c r="S83" s="4" t="n"/>
+      <c r="T83" s="4" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n"/>
@@ -2464,6 +2559,7 @@
       <c r="Q84" s="4" t="n"/>
       <c r="R84" s="4" t="n"/>
       <c r="S84" s="4" t="n"/>
+      <c r="T84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n"/>
@@ -2485,6 +2581,7 @@
       <c r="Q85" s="4" t="n"/>
       <c r="R85" s="4" t="n"/>
       <c r="S85" s="4" t="n"/>
+      <c r="T85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="n"/>
@@ -2506,6 +2603,7 @@
       <c r="Q86" s="4" t="n"/>
       <c r="R86" s="4" t="n"/>
       <c r="S86" s="4" t="n"/>
+      <c r="T86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n"/>
@@ -2527,6 +2625,7 @@
       <c r="Q87" s="4" t="n"/>
       <c r="R87" s="4" t="n"/>
       <c r="S87" s="4" t="n"/>
+      <c r="T87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="n"/>
@@ -2548,6 +2647,7 @@
       <c r="Q88" s="4" t="n"/>
       <c r="R88" s="4" t="n"/>
       <c r="S88" s="4" t="n"/>
+      <c r="T88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n"/>
@@ -2569,6 +2669,7 @@
       <c r="Q89" s="4" t="n"/>
       <c r="R89" s="4" t="n"/>
       <c r="S89" s="4" t="n"/>
+      <c r="T89" s="4" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n"/>
@@ -2590,6 +2691,7 @@
       <c r="Q90" s="4" t="n"/>
       <c r="R90" s="4" t="n"/>
       <c r="S90" s="4" t="n"/>
+      <c r="T90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n"/>
@@ -2611,6 +2713,7 @@
       <c r="Q91" s="4" t="n"/>
       <c r="R91" s="4" t="n"/>
       <c r="S91" s="4" t="n"/>
+      <c r="T91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="n"/>
@@ -2632,6 +2735,7 @@
       <c r="Q92" s="4" t="n"/>
       <c r="R92" s="4" t="n"/>
       <c r="S92" s="4" t="n"/>
+      <c r="T92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n"/>
@@ -2653,6 +2757,7 @@
       <c r="Q93" s="4" t="n"/>
       <c r="R93" s="4" t="n"/>
       <c r="S93" s="4" t="n"/>
+      <c r="T93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="n"/>
@@ -2674,6 +2779,7 @@
       <c r="Q94" s="4" t="n"/>
       <c r="R94" s="4" t="n"/>
       <c r="S94" s="4" t="n"/>
+      <c r="T94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n"/>
@@ -2695,6 +2801,7 @@
       <c r="Q95" s="4" t="n"/>
       <c r="R95" s="4" t="n"/>
       <c r="S95" s="4" t="n"/>
+      <c r="T95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="n"/>
@@ -2716,6 +2823,7 @@
       <c r="Q96" s="4" t="n"/>
       <c r="R96" s="4" t="n"/>
       <c r="S96" s="4" t="n"/>
+      <c r="T96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n"/>
@@ -2737,6 +2845,7 @@
       <c r="Q97" s="4" t="n"/>
       <c r="R97" s="4" t="n"/>
       <c r="S97" s="4" t="n"/>
+      <c r="T97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="n"/>
@@ -2758,6 +2867,7 @@
       <c r="Q98" s="4" t="n"/>
       <c r="R98" s="4" t="n"/>
       <c r="S98" s="4" t="n"/>
+      <c r="T98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n"/>
@@ -2779,6 +2889,7 @@
       <c r="Q99" s="4" t="n"/>
       <c r="R99" s="4" t="n"/>
       <c r="S99" s="4" t="n"/>
+      <c r="T99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="n"/>
@@ -2800,6 +2911,7 @@
       <c r="Q100" s="4" t="n"/>
       <c r="R100" s="4" t="n"/>
       <c r="S100" s="4" t="n"/>
+      <c r="T100" s="4" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n"/>
@@ -2821,6 +2933,7 @@
       <c r="Q101" s="4" t="n"/>
       <c r="R101" s="4" t="n"/>
       <c r="S101" s="4" t="n"/>
+      <c r="T101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="n"/>
@@ -2842,6 +2955,7 @@
       <c r="Q102" s="4" t="n"/>
       <c r="R102" s="4" t="n"/>
       <c r="S102" s="4" t="n"/>
+      <c r="T102" s="4" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="n"/>
@@ -2863,6 +2977,7 @@
       <c r="Q103" s="4" t="n"/>
       <c r="R103" s="4" t="n"/>
       <c r="S103" s="4" t="n"/>
+      <c r="T103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="n"/>
@@ -2884,6 +2999,7 @@
       <c r="Q104" s="4" t="n"/>
       <c r="R104" s="4" t="n"/>
       <c r="S104" s="4" t="n"/>
+      <c r="T104" s="4" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="n"/>
@@ -2905,6 +3021,7 @@
       <c r="Q105" s="4" t="n"/>
       <c r="R105" s="4" t="n"/>
       <c r="S105" s="4" t="n"/>
+      <c r="T105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="n"/>
@@ -2926,6 +3043,7 @@
       <c r="Q106" s="4" t="n"/>
       <c r="R106" s="4" t="n"/>
       <c r="S106" s="4" t="n"/>
+      <c r="T106" s="4" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n"/>
@@ -2947,6 +3065,7 @@
       <c r="Q107" s="4" t="n"/>
       <c r="R107" s="4" t="n"/>
       <c r="S107" s="4" t="n"/>
+      <c r="T107" s="4" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n"/>
@@ -2968,6 +3087,7 @@
       <c r="Q108" s="4" t="n"/>
       <c r="R108" s="4" t="n"/>
       <c r="S108" s="4" t="n"/>
+      <c r="T108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="n"/>
@@ -2989,6 +3109,7 @@
       <c r="Q109" s="4" t="n"/>
       <c r="R109" s="4" t="n"/>
       <c r="S109" s="4" t="n"/>
+      <c r="T109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n"/>
@@ -3010,6 +3131,7 @@
       <c r="Q110" s="4" t="n"/>
       <c r="R110" s="4" t="n"/>
       <c r="S110" s="4" t="n"/>
+      <c r="T110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n"/>
@@ -3031,6 +3153,7 @@
       <c r="Q111" s="4" t="n"/>
       <c r="R111" s="4" t="n"/>
       <c r="S111" s="4" t="n"/>
+      <c r="T111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n"/>
@@ -3052,6 +3175,7 @@
       <c r="Q112" s="4" t="n"/>
       <c r="R112" s="4" t="n"/>
       <c r="S112" s="4" t="n"/>
+      <c r="T112" s="4" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n"/>
@@ -3073,6 +3197,7 @@
       <c r="Q113" s="4" t="n"/>
       <c r="R113" s="4" t="n"/>
       <c r="S113" s="4" t="n"/>
+      <c r="T113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="n"/>
@@ -3094,6 +3219,7 @@
       <c r="Q114" s="4" t="n"/>
       <c r="R114" s="4" t="n"/>
       <c r="S114" s="4" t="n"/>
+      <c r="T114" s="4" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="n"/>
@@ -3115,6 +3241,7 @@
       <c r="Q115" s="4" t="n"/>
       <c r="R115" s="4" t="n"/>
       <c r="S115" s="4" t="n"/>
+      <c r="T115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="n"/>
@@ -3136,6 +3263,7 @@
       <c r="Q116" s="4" t="n"/>
       <c r="R116" s="4" t="n"/>
       <c r="S116" s="4" t="n"/>
+      <c r="T116" s="4" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n"/>
@@ -3157,6 +3285,7 @@
       <c r="Q117" s="4" t="n"/>
       <c r="R117" s="4" t="n"/>
       <c r="S117" s="4" t="n"/>
+      <c r="T117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="n"/>
@@ -3178,6 +3307,7 @@
       <c r="Q118" s="4" t="n"/>
       <c r="R118" s="4" t="n"/>
       <c r="S118" s="4" t="n"/>
+      <c r="T118" s="4" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="n"/>
@@ -3199,6 +3329,7 @@
       <c r="Q119" s="4" t="n"/>
       <c r="R119" s="4" t="n"/>
       <c r="S119" s="4" t="n"/>
+      <c r="T119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="n"/>
@@ -3220,6 +3351,7 @@
       <c r="Q120" s="4" t="n"/>
       <c r="R120" s="4" t="n"/>
       <c r="S120" s="4" t="n"/>
+      <c r="T120" s="4" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="n"/>
@@ -3241,6 +3373,7 @@
       <c r="Q121" s="4" t="n"/>
       <c r="R121" s="4" t="n"/>
       <c r="S121" s="4" t="n"/>
+      <c r="T121" s="4" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="n"/>
@@ -3262,6 +3395,7 @@
       <c r="Q122" s="4" t="n"/>
       <c r="R122" s="4" t="n"/>
       <c r="S122" s="4" t="n"/>
+      <c r="T122" s="4" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="n"/>
@@ -3283,6 +3417,7 @@
       <c r="Q123" s="4" t="n"/>
       <c r="R123" s="4" t="n"/>
       <c r="S123" s="4" t="n"/>
+      <c r="T123" s="4" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="n"/>
@@ -3304,6 +3439,7 @@
       <c r="Q124" s="4" t="n"/>
       <c r="R124" s="4" t="n"/>
       <c r="S124" s="4" t="n"/>
+      <c r="T124" s="4" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="n"/>
@@ -3325,6 +3461,7 @@
       <c r="Q125" s="4" t="n"/>
       <c r="R125" s="4" t="n"/>
       <c r="S125" s="4" t="n"/>
+      <c r="T125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="n"/>
@@ -3346,6 +3483,7 @@
       <c r="Q126" s="4" t="n"/>
       <c r="R126" s="4" t="n"/>
       <c r="S126" s="4" t="n"/>
+      <c r="T126" s="4" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="n"/>
@@ -3367,6 +3505,7 @@
       <c r="Q127" s="4" t="n"/>
       <c r="R127" s="4" t="n"/>
       <c r="S127" s="4" t="n"/>
+      <c r="T127" s="4" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="n"/>
@@ -3388,6 +3527,7 @@
       <c r="Q128" s="4" t="n"/>
       <c r="R128" s="4" t="n"/>
       <c r="S128" s="4" t="n"/>
+      <c r="T128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="n"/>
@@ -3409,6 +3549,7 @@
       <c r="Q129" s="4" t="n"/>
       <c r="R129" s="4" t="n"/>
       <c r="S129" s="4" t="n"/>
+      <c r="T129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="n"/>
@@ -3430,6 +3571,7 @@
       <c r="Q130" s="4" t="n"/>
       <c r="R130" s="4" t="n"/>
       <c r="S130" s="4" t="n"/>
+      <c r="T130" s="4" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="n"/>
@@ -3451,6 +3593,7 @@
       <c r="Q131" s="4" t="n"/>
       <c r="R131" s="4" t="n"/>
       <c r="S131" s="4" t="n"/>
+      <c r="T131" s="4" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="n"/>
@@ -3472,6 +3615,7 @@
       <c r="Q132" s="4" t="n"/>
       <c r="R132" s="4" t="n"/>
       <c r="S132" s="4" t="n"/>
+      <c r="T132" s="4" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="n"/>
@@ -3493,6 +3637,7 @@
       <c r="Q133" s="4" t="n"/>
       <c r="R133" s="4" t="n"/>
       <c r="S133" s="4" t="n"/>
+      <c r="T133" s="4" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="n"/>
@@ -3514,6 +3659,7 @@
       <c r="Q134" s="4" t="n"/>
       <c r="R134" s="4" t="n"/>
       <c r="S134" s="4" t="n"/>
+      <c r="T134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="n"/>
@@ -3535,6 +3681,7 @@
       <c r="Q135" s="4" t="n"/>
       <c r="R135" s="4" t="n"/>
       <c r="S135" s="4" t="n"/>
+      <c r="T135" s="4" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="n"/>
@@ -3556,6 +3703,7 @@
       <c r="Q136" s="4" t="n"/>
       <c r="R136" s="4" t="n"/>
       <c r="S136" s="4" t="n"/>
+      <c r="T136" s="4" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n"/>
@@ -3577,6 +3725,7 @@
       <c r="Q137" s="4" t="n"/>
       <c r="R137" s="4" t="n"/>
       <c r="S137" s="4" t="n"/>
+      <c r="T137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="n"/>
@@ -3598,6 +3747,7 @@
       <c r="Q138" s="4" t="n"/>
       <c r="R138" s="4" t="n"/>
       <c r="S138" s="4" t="n"/>
+      <c r="T138" s="4" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="n"/>
@@ -3619,6 +3769,7 @@
       <c r="Q139" s="4" t="n"/>
       <c r="R139" s="4" t="n"/>
       <c r="S139" s="4" t="n"/>
+      <c r="T139" s="4" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="n"/>
@@ -3640,6 +3791,7 @@
       <c r="Q140" s="4" t="n"/>
       <c r="R140" s="4" t="n"/>
       <c r="S140" s="4" t="n"/>
+      <c r="T140" s="4" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="n"/>
@@ -3661,6 +3813,7 @@
       <c r="Q141" s="4" t="n"/>
       <c r="R141" s="4" t="n"/>
       <c r="S141" s="4" t="n"/>
+      <c r="T141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="n"/>
@@ -3682,6 +3835,7 @@
       <c r="Q142" s="4" t="n"/>
       <c r="R142" s="4" t="n"/>
       <c r="S142" s="4" t="n"/>
+      <c r="T142" s="4" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="n"/>
@@ -3703,6 +3857,7 @@
       <c r="Q143" s="4" t="n"/>
       <c r="R143" s="4" t="n"/>
       <c r="S143" s="4" t="n"/>
+      <c r="T143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="n"/>
@@ -3724,6 +3879,7 @@
       <c r="Q144" s="4" t="n"/>
       <c r="R144" s="4" t="n"/>
       <c r="S144" s="4" t="n"/>
+      <c r="T144" s="4" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="n"/>
@@ -3745,6 +3901,7 @@
       <c r="Q145" s="4" t="n"/>
       <c r="R145" s="4" t="n"/>
       <c r="S145" s="4" t="n"/>
+      <c r="T145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="n"/>
@@ -3766,6 +3923,7 @@
       <c r="Q146" s="4" t="n"/>
       <c r="R146" s="4" t="n"/>
       <c r="S146" s="4" t="n"/>
+      <c r="T146" s="4" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="n"/>
@@ -3787,6 +3945,7 @@
       <c r="Q147" s="4" t="n"/>
       <c r="R147" s="4" t="n"/>
       <c r="S147" s="4" t="n"/>
+      <c r="T147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="n"/>
@@ -3808,6 +3967,7 @@
       <c r="Q148" s="4" t="n"/>
       <c r="R148" s="4" t="n"/>
       <c r="S148" s="4" t="n"/>
+      <c r="T148" s="4" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="n"/>
@@ -3829,6 +3989,7 @@
       <c r="Q149" s="4" t="n"/>
       <c r="R149" s="4" t="n"/>
       <c r="S149" s="4" t="n"/>
+      <c r="T149" s="4" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="n"/>
@@ -3850,6 +4011,7 @@
       <c r="Q150" s="4" t="n"/>
       <c r="R150" s="4" t="n"/>
       <c r="S150" s="4" t="n"/>
+      <c r="T150" s="4" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="n"/>
@@ -3871,6 +4033,7 @@
       <c r="Q151" s="4" t="n"/>
       <c r="R151" s="4" t="n"/>
       <c r="S151" s="4" t="n"/>
+      <c r="T151" s="4" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="n"/>
@@ -3892,6 +4055,7 @@
       <c r="Q152" s="4" t="n"/>
       <c r="R152" s="4" t="n"/>
       <c r="S152" s="4" t="n"/>
+      <c r="T152" s="4" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="n"/>
@@ -3913,6 +4077,7 @@
       <c r="Q153" s="4" t="n"/>
       <c r="R153" s="4" t="n"/>
       <c r="S153" s="4" t="n"/>
+      <c r="T153" s="4" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="n"/>
@@ -3934,6 +4099,7 @@
       <c r="Q154" s="4" t="n"/>
       <c r="R154" s="4" t="n"/>
       <c r="S154" s="4" t="n"/>
+      <c r="T154" s="4" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="n"/>
@@ -3955,6 +4121,7 @@
       <c r="Q155" s="4" t="n"/>
       <c r="R155" s="4" t="n"/>
       <c r="S155" s="4" t="n"/>
+      <c r="T155" s="4" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="n"/>
@@ -3976,6 +4143,7 @@
       <c r="Q156" s="4" t="n"/>
       <c r="R156" s="4" t="n"/>
       <c r="S156" s="4" t="n"/>
+      <c r="T156" s="4" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="n"/>
@@ -3997,6 +4165,7 @@
       <c r="Q157" s="4" t="n"/>
       <c r="R157" s="4" t="n"/>
       <c r="S157" s="4" t="n"/>
+      <c r="T157" s="4" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="n"/>
@@ -4018,6 +4187,7 @@
       <c r="Q158" s="4" t="n"/>
       <c r="R158" s="4" t="n"/>
       <c r="S158" s="4" t="n"/>
+      <c r="T158" s="4" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n"/>
@@ -4039,6 +4209,7 @@
       <c r="Q159" s="4" t="n"/>
       <c r="R159" s="4" t="n"/>
       <c r="S159" s="4" t="n"/>
+      <c r="T159" s="4" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="n"/>
@@ -4060,6 +4231,7 @@
       <c r="Q160" s="4" t="n"/>
       <c r="R160" s="4" t="n"/>
       <c r="S160" s="4" t="n"/>
+      <c r="T160" s="4" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="n"/>
@@ -4081,6 +4253,7 @@
       <c r="Q161" s="4" t="n"/>
       <c r="R161" s="4" t="n"/>
       <c r="S161" s="4" t="n"/>
+      <c r="T161" s="4" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="n"/>
@@ -4102,6 +4275,7 @@
       <c r="Q162" s="4" t="n"/>
       <c r="R162" s="4" t="n"/>
       <c r="S162" s="4" t="n"/>
+      <c r="T162" s="4" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="n"/>
@@ -4123,6 +4297,7 @@
       <c r="Q163" s="4" t="n"/>
       <c r="R163" s="4" t="n"/>
       <c r="S163" s="4" t="n"/>
+      <c r="T163" s="4" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="n"/>
@@ -4144,6 +4319,7 @@
       <c r="Q164" s="4" t="n"/>
       <c r="R164" s="4" t="n"/>
       <c r="S164" s="4" t="n"/>
+      <c r="T164" s="4" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="n"/>
@@ -4165,6 +4341,7 @@
       <c r="Q165" s="4" t="n"/>
       <c r="R165" s="4" t="n"/>
       <c r="S165" s="4" t="n"/>
+      <c r="T165" s="4" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="n"/>
@@ -4186,6 +4363,7 @@
       <c r="Q166" s="4" t="n"/>
       <c r="R166" s="4" t="n"/>
       <c r="S166" s="4" t="n"/>
+      <c r="T166" s="4" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="n"/>
@@ -4207,6 +4385,7 @@
       <c r="Q167" s="4" t="n"/>
       <c r="R167" s="4" t="n"/>
       <c r="S167" s="4" t="n"/>
+      <c r="T167" s="4" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="n"/>
@@ -4228,6 +4407,7 @@
       <c r="Q168" s="4" t="n"/>
       <c r="R168" s="4" t="n"/>
       <c r="S168" s="4" t="n"/>
+      <c r="T168" s="4" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="n"/>
@@ -4249,6 +4429,7 @@
       <c r="Q169" s="4" t="n"/>
       <c r="R169" s="4" t="n"/>
       <c r="S169" s="4" t="n"/>
+      <c r="T169" s="4" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="n"/>
@@ -4270,6 +4451,7 @@
       <c r="Q170" s="4" t="n"/>
       <c r="R170" s="4" t="n"/>
       <c r="S170" s="4" t="n"/>
+      <c r="T170" s="4" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="n"/>
@@ -4291,6 +4473,7 @@
       <c r="Q171" s="4" t="n"/>
       <c r="R171" s="4" t="n"/>
       <c r="S171" s="4" t="n"/>
+      <c r="T171" s="4" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="n"/>
@@ -4312,6 +4495,7 @@
       <c r="Q172" s="4" t="n"/>
       <c r="R172" s="4" t="n"/>
       <c r="S172" s="4" t="n"/>
+      <c r="T172" s="4" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="n"/>
@@ -4333,6 +4517,7 @@
       <c r="Q173" s="4" t="n"/>
       <c r="R173" s="4" t="n"/>
       <c r="S173" s="4" t="n"/>
+      <c r="T173" s="4" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n"/>
@@ -4354,6 +4539,7 @@
       <c r="Q174" s="4" t="n"/>
       <c r="R174" s="4" t="n"/>
       <c r="S174" s="4" t="n"/>
+      <c r="T174" s="4" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="n"/>
@@ -4375,6 +4561,7 @@
       <c r="Q175" s="4" t="n"/>
       <c r="R175" s="4" t="n"/>
       <c r="S175" s="4" t="n"/>
+      <c r="T175" s="4" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="n"/>
@@ -4396,6 +4583,7 @@
       <c r="Q176" s="4" t="n"/>
       <c r="R176" s="4" t="n"/>
       <c r="S176" s="4" t="n"/>
+      <c r="T176" s="4" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="n"/>
@@ -4417,6 +4605,7 @@
       <c r="Q177" s="4" t="n"/>
       <c r="R177" s="4" t="n"/>
       <c r="S177" s="4" t="n"/>
+      <c r="T177" s="4" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="n"/>
@@ -4438,6 +4627,7 @@
       <c r="Q178" s="4" t="n"/>
       <c r="R178" s="4" t="n"/>
       <c r="S178" s="4" t="n"/>
+      <c r="T178" s="4" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="n"/>
@@ -4459,6 +4649,7 @@
       <c r="Q179" s="4" t="n"/>
       <c r="R179" s="4" t="n"/>
       <c r="S179" s="4" t="n"/>
+      <c r="T179" s="4" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="n"/>
@@ -4480,6 +4671,7 @@
       <c r="Q180" s="4" t="n"/>
       <c r="R180" s="4" t="n"/>
       <c r="S180" s="4" t="n"/>
+      <c r="T180" s="4" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="n"/>
@@ -4501,6 +4693,7 @@
       <c r="Q181" s="4" t="n"/>
       <c r="R181" s="4" t="n"/>
       <c r="S181" s="4" t="n"/>
+      <c r="T181" s="4" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="n"/>
@@ -4522,6 +4715,7 @@
       <c r="Q182" s="4" t="n"/>
       <c r="R182" s="4" t="n"/>
       <c r="S182" s="4" t="n"/>
+      <c r="T182" s="4" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="n"/>
@@ -4543,6 +4737,7 @@
       <c r="Q183" s="4" t="n"/>
       <c r="R183" s="4" t="n"/>
       <c r="S183" s="4" t="n"/>
+      <c r="T183" s="4" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="n"/>
@@ -4564,6 +4759,7 @@
       <c r="Q184" s="4" t="n"/>
       <c r="R184" s="4" t="n"/>
       <c r="S184" s="4" t="n"/>
+      <c r="T184" s="4" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="n"/>
@@ -4585,6 +4781,7 @@
       <c r="Q185" s="4" t="n"/>
       <c r="R185" s="4" t="n"/>
       <c r="S185" s="4" t="n"/>
+      <c r="T185" s="4" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="n"/>
@@ -4606,6 +4803,7 @@
       <c r="Q186" s="4" t="n"/>
       <c r="R186" s="4" t="n"/>
       <c r="S186" s="4" t="n"/>
+      <c r="T186" s="4" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="n"/>
@@ -4627,6 +4825,7 @@
       <c r="Q187" s="4" t="n"/>
       <c r="R187" s="4" t="n"/>
       <c r="S187" s="4" t="n"/>
+      <c r="T187" s="4" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="n"/>
@@ -4648,6 +4847,7 @@
       <c r="Q188" s="4" t="n"/>
       <c r="R188" s="4" t="n"/>
       <c r="S188" s="4" t="n"/>
+      <c r="T188" s="4" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="n"/>
@@ -4669,6 +4869,7 @@
       <c r="Q189" s="4" t="n"/>
       <c r="R189" s="4" t="n"/>
       <c r="S189" s="4" t="n"/>
+      <c r="T189" s="4" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="n"/>
@@ -4690,6 +4891,7 @@
       <c r="Q190" s="4" t="n"/>
       <c r="R190" s="4" t="n"/>
       <c r="S190" s="4" t="n"/>
+      <c r="T190" s="4" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="n"/>
@@ -4711,6 +4913,7 @@
       <c r="Q191" s="4" t="n"/>
       <c r="R191" s="4" t="n"/>
       <c r="S191" s="4" t="n"/>
+      <c r="T191" s="4" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="n"/>
@@ -4732,6 +4935,7 @@
       <c r="Q192" s="4" t="n"/>
       <c r="R192" s="4" t="n"/>
       <c r="S192" s="4" t="n"/>
+      <c r="T192" s="4" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="4" t="n"/>
@@ -4753,6 +4957,7 @@
       <c r="Q193" s="4" t="n"/>
       <c r="R193" s="4" t="n"/>
       <c r="S193" s="4" t="n"/>
+      <c r="T193" s="4" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="n"/>
@@ -4774,6 +4979,7 @@
       <c r="Q194" s="4" t="n"/>
       <c r="R194" s="4" t="n"/>
       <c r="S194" s="4" t="n"/>
+      <c r="T194" s="4" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="n"/>
@@ -4795,6 +5001,7 @@
       <c r="Q195" s="4" t="n"/>
       <c r="R195" s="4" t="n"/>
       <c r="S195" s="4" t="n"/>
+      <c r="T195" s="4" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="n"/>
@@ -4816,6 +5023,7 @@
       <c r="Q196" s="4" t="n"/>
       <c r="R196" s="4" t="n"/>
       <c r="S196" s="4" t="n"/>
+      <c r="T196" s="4" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="n"/>
@@ -4837,6 +5045,7 @@
       <c r="Q197" s="4" t="n"/>
       <c r="R197" s="4" t="n"/>
       <c r="S197" s="4" t="n"/>
+      <c r="T197" s="4" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="n"/>
@@ -4858,6 +5067,7 @@
       <c r="Q198" s="4" t="n"/>
       <c r="R198" s="4" t="n"/>
       <c r="S198" s="4" t="n"/>
+      <c r="T198" s="4" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="4" t="n"/>
@@ -4879,6 +5089,7 @@
       <c r="Q199" s="4" t="n"/>
       <c r="R199" s="4" t="n"/>
       <c r="S199" s="4" t="n"/>
+      <c r="T199" s="4" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="4" t="n"/>
@@ -4900,6 +5111,7 @@
       <c r="Q200" s="4" t="n"/>
       <c r="R200" s="4" t="n"/>
       <c r="S200" s="4" t="n"/>
+      <c r="T200" s="4" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="n"/>
@@ -4921,6 +5133,7 @@
       <c r="Q201" s="4" t="n"/>
       <c r="R201" s="4" t="n"/>
       <c r="S201" s="4" t="n"/>
+      <c r="T201" s="4" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="4" t="n"/>
@@ -4942,6 +5155,7 @@
       <c r="Q202" s="4" t="n"/>
       <c r="R202" s="4" t="n"/>
       <c r="S202" s="4" t="n"/>
+      <c r="T202" s="4" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="4" t="n"/>
@@ -4963,6 +5177,7 @@
       <c r="Q203" s="4" t="n"/>
       <c r="R203" s="4" t="n"/>
       <c r="S203" s="4" t="n"/>
+      <c r="T203" s="4" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="4" t="n"/>
@@ -4984,6 +5199,7 @@
       <c r="Q204" s="4" t="n"/>
       <c r="R204" s="4" t="n"/>
       <c r="S204" s="4" t="n"/>
+      <c r="T204" s="4" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="4" t="n"/>
@@ -5005,6 +5221,7 @@
       <c r="Q205" s="4" t="n"/>
       <c r="R205" s="4" t="n"/>
       <c r="S205" s="4" t="n"/>
+      <c r="T205" s="4" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="4" t="n"/>
@@ -5026,6 +5243,7 @@
       <c r="Q206" s="4" t="n"/>
       <c r="R206" s="4" t="n"/>
       <c r="S206" s="4" t="n"/>
+      <c r="T206" s="4" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="n"/>
@@ -5047,6 +5265,7 @@
       <c r="Q207" s="4" t="n"/>
       <c r="R207" s="4" t="n"/>
       <c r="S207" s="4" t="n"/>
+      <c r="T207" s="4" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="4" t="n"/>
@@ -5068,6 +5287,7 @@
       <c r="Q208" s="4" t="n"/>
       <c r="R208" s="4" t="n"/>
       <c r="S208" s="4" t="n"/>
+      <c r="T208" s="4" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="4" t="n"/>
@@ -5089,6 +5309,7 @@
       <c r="Q209" s="4" t="n"/>
       <c r="R209" s="4" t="n"/>
       <c r="S209" s="4" t="n"/>
+      <c r="T209" s="4" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="n"/>
@@ -5110,6 +5331,7 @@
       <c r="Q210" s="4" t="n"/>
       <c r="R210" s="4" t="n"/>
       <c r="S210" s="4" t="n"/>
+      <c r="T210" s="4" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="n"/>
@@ -5131,6 +5353,7 @@
       <c r="Q211" s="4" t="n"/>
       <c r="R211" s="4" t="n"/>
       <c r="S211" s="4" t="n"/>
+      <c r="T211" s="4" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="n"/>
@@ -5152,6 +5375,7 @@
       <c r="Q212" s="4" t="n"/>
       <c r="R212" s="4" t="n"/>
       <c r="S212" s="4" t="n"/>
+      <c r="T212" s="4" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="4" t="n"/>
@@ -5173,6 +5397,7 @@
       <c r="Q213" s="4" t="n"/>
       <c r="R213" s="4" t="n"/>
       <c r="S213" s="4" t="n"/>
+      <c r="T213" s="4" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="n"/>
@@ -5194,6 +5419,7 @@
       <c r="Q214" s="4" t="n"/>
       <c r="R214" s="4" t="n"/>
       <c r="S214" s="4" t="n"/>
+      <c r="T214" s="4" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="4" t="n"/>
@@ -5215,6 +5441,7 @@
       <c r="Q215" s="4" t="n"/>
       <c r="R215" s="4" t="n"/>
       <c r="S215" s="4" t="n"/>
+      <c r="T215" s="4" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="4" t="n"/>
@@ -5236,6 +5463,7 @@
       <c r="Q216" s="4" t="n"/>
       <c r="R216" s="4" t="n"/>
       <c r="S216" s="4" t="n"/>
+      <c r="T216" s="4" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="4" t="n"/>
@@ -5257,6 +5485,7 @@
       <c r="Q217" s="4" t="n"/>
       <c r="R217" s="4" t="n"/>
       <c r="S217" s="4" t="n"/>
+      <c r="T217" s="4" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="4" t="n"/>
@@ -5278,6 +5507,7 @@
       <c r="Q218" s="4" t="n"/>
       <c r="R218" s="4" t="n"/>
       <c r="S218" s="4" t="n"/>
+      <c r="T218" s="4" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="n"/>
@@ -5299,6 +5529,7 @@
       <c r="Q219" s="4" t="n"/>
       <c r="R219" s="4" t="n"/>
       <c r="S219" s="4" t="n"/>
+      <c r="T219" s="4" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="4" t="n"/>
@@ -5320,6 +5551,7 @@
       <c r="Q220" s="4" t="n"/>
       <c r="R220" s="4" t="n"/>
       <c r="S220" s="4" t="n"/>
+      <c r="T220" s="4" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="4" t="n"/>
@@ -5341,6 +5573,7 @@
       <c r="Q221" s="4" t="n"/>
       <c r="R221" s="4" t="n"/>
       <c r="S221" s="4" t="n"/>
+      <c r="T221" s="4" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="4" t="n"/>
@@ -5362,6 +5595,7 @@
       <c r="Q222" s="4" t="n"/>
       <c r="R222" s="4" t="n"/>
       <c r="S222" s="4" t="n"/>
+      <c r="T222" s="4" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="4" t="n"/>
@@ -5383,6 +5617,7 @@
       <c r="Q223" s="4" t="n"/>
       <c r="R223" s="4" t="n"/>
       <c r="S223" s="4" t="n"/>
+      <c r="T223" s="4" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="4" t="n"/>
@@ -5404,6 +5639,7 @@
       <c r="Q224" s="4" t="n"/>
       <c r="R224" s="4" t="n"/>
       <c r="S224" s="4" t="n"/>
+      <c r="T224" s="4" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="4" t="n"/>
@@ -5425,6 +5661,7 @@
       <c r="Q225" s="4" t="n"/>
       <c r="R225" s="4" t="n"/>
       <c r="S225" s="4" t="n"/>
+      <c r="T225" s="4" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="4" t="n"/>
@@ -5446,6 +5683,7 @@
       <c r="Q226" s="4" t="n"/>
       <c r="R226" s="4" t="n"/>
       <c r="S226" s="4" t="n"/>
+      <c r="T226" s="4" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="n"/>
@@ -5467,6 +5705,7 @@
       <c r="Q227" s="4" t="n"/>
       <c r="R227" s="4" t="n"/>
       <c r="S227" s="4" t="n"/>
+      <c r="T227" s="4" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="4" t="n"/>
@@ -5488,6 +5727,7 @@
       <c r="Q228" s="4" t="n"/>
       <c r="R228" s="4" t="n"/>
       <c r="S228" s="4" t="n"/>
+      <c r="T228" s="4" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="4" t="n"/>
@@ -5509,6 +5749,7 @@
       <c r="Q229" s="4" t="n"/>
       <c r="R229" s="4" t="n"/>
       <c r="S229" s="4" t="n"/>
+      <c r="T229" s="4" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="4" t="n"/>
@@ -5530,6 +5771,7 @@
       <c r="Q230" s="4" t="n"/>
       <c r="R230" s="4" t="n"/>
       <c r="S230" s="4" t="n"/>
+      <c r="T230" s="4" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="n"/>
@@ -5551,6 +5793,7 @@
       <c r="Q231" s="4" t="n"/>
       <c r="R231" s="4" t="n"/>
       <c r="S231" s="4" t="n"/>
+      <c r="T231" s="4" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="n"/>
@@ -5572,6 +5815,7 @@
       <c r="Q232" s="4" t="n"/>
       <c r="R232" s="4" t="n"/>
       <c r="S232" s="4" t="n"/>
+      <c r="T232" s="4" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="4" t="n"/>
@@ -5593,6 +5837,7 @@
       <c r="Q233" s="4" t="n"/>
       <c r="R233" s="4" t="n"/>
       <c r="S233" s="4" t="n"/>
+      <c r="T233" s="4" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="n"/>
@@ -5614,6 +5859,7 @@
       <c r="Q234" s="4" t="n"/>
       <c r="R234" s="4" t="n"/>
       <c r="S234" s="4" t="n"/>
+      <c r="T234" s="4" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="4" t="n"/>
@@ -5635,6 +5881,7 @@
       <c r="Q235" s="4" t="n"/>
       <c r="R235" s="4" t="n"/>
       <c r="S235" s="4" t="n"/>
+      <c r="T235" s="4" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="4" t="n"/>
@@ -5656,6 +5903,7 @@
       <c r="Q236" s="4" t="n"/>
       <c r="R236" s="4" t="n"/>
       <c r="S236" s="4" t="n"/>
+      <c r="T236" s="4" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="4" t="n"/>
@@ -5677,6 +5925,7 @@
       <c r="Q237" s="4" t="n"/>
       <c r="R237" s="4" t="n"/>
       <c r="S237" s="4" t="n"/>
+      <c r="T237" s="4" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="4" t="n"/>
@@ -5698,6 +5947,7 @@
       <c r="Q238" s="4" t="n"/>
       <c r="R238" s="4" t="n"/>
       <c r="S238" s="4" t="n"/>
+      <c r="T238" s="4" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="4" t="n"/>
@@ -5719,6 +5969,7 @@
       <c r="Q239" s="4" t="n"/>
       <c r="R239" s="4" t="n"/>
       <c r="S239" s="4" t="n"/>
+      <c r="T239" s="4" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="4" t="n"/>
@@ -5740,6 +5991,7 @@
       <c r="Q240" s="4" t="n"/>
       <c r="R240" s="4" t="n"/>
       <c r="S240" s="4" t="n"/>
+      <c r="T240" s="4" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="4" t="n"/>
@@ -5761,6 +6013,7 @@
       <c r="Q241" s="4" t="n"/>
       <c r="R241" s="4" t="n"/>
       <c r="S241" s="4" t="n"/>
+      <c r="T241" s="4" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="4" t="n"/>
@@ -5782,6 +6035,7 @@
       <c r="Q242" s="4" t="n"/>
       <c r="R242" s="4" t="n"/>
       <c r="S242" s="4" t="n"/>
+      <c r="T242" s="4" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="4" t="n"/>
@@ -5803,6 +6057,7 @@
       <c r="Q243" s="4" t="n"/>
       <c r="R243" s="4" t="n"/>
       <c r="S243" s="4" t="n"/>
+      <c r="T243" s="4" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="n"/>
@@ -5824,6 +6079,7 @@
       <c r="Q244" s="4" t="n"/>
       <c r="R244" s="4" t="n"/>
       <c r="S244" s="4" t="n"/>
+      <c r="T244" s="4" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="4" t="n"/>
@@ -5845,6 +6101,7 @@
       <c r="Q245" s="4" t="n"/>
       <c r="R245" s="4" t="n"/>
       <c r="S245" s="4" t="n"/>
+      <c r="T245" s="4" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="4" t="n"/>
@@ -5866,6 +6123,7 @@
       <c r="Q246" s="4" t="n"/>
       <c r="R246" s="4" t="n"/>
       <c r="S246" s="4" t="n"/>
+      <c r="T246" s="4" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="4" t="n"/>
@@ -5887,6 +6145,7 @@
       <c r="Q247" s="4" t="n"/>
       <c r="R247" s="4" t="n"/>
       <c r="S247" s="4" t="n"/>
+      <c r="T247" s="4" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="4" t="n"/>
@@ -5908,6 +6167,7 @@
       <c r="Q248" s="4" t="n"/>
       <c r="R248" s="4" t="n"/>
       <c r="S248" s="4" t="n"/>
+      <c r="T248" s="4" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="4" t="n"/>
@@ -5929,6 +6189,7 @@
       <c r="Q249" s="4" t="n"/>
       <c r="R249" s="4" t="n"/>
       <c r="S249" s="4" t="n"/>
+      <c r="T249" s="4" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="4" t="n"/>
@@ -5950,6 +6211,7 @@
       <c r="Q250" s="4" t="n"/>
       <c r="R250" s="4" t="n"/>
       <c r="S250" s="4" t="n"/>
+      <c r="T250" s="4" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="4" t="n"/>
@@ -5971,6 +6233,7 @@
       <c r="Q251" s="4" t="n"/>
       <c r="R251" s="4" t="n"/>
       <c r="S251" s="4" t="n"/>
+      <c r="T251" s="4" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="4" t="n"/>
@@ -5992,6 +6255,7 @@
       <c r="Q252" s="4" t="n"/>
       <c r="R252" s="4" t="n"/>
       <c r="S252" s="4" t="n"/>
+      <c r="T252" s="4" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="4" t="n"/>
@@ -6013,6 +6277,7 @@
       <c r="Q253" s="4" t="n"/>
       <c r="R253" s="4" t="n"/>
       <c r="S253" s="4" t="n"/>
+      <c r="T253" s="4" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="n"/>
@@ -6034,6 +6299,7 @@
       <c r="Q254" s="4" t="n"/>
       <c r="R254" s="4" t="n"/>
       <c r="S254" s="4" t="n"/>
+      <c r="T254" s="4" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="4" t="n"/>
@@ -6055,6 +6321,7 @@
       <c r="Q255" s="4" t="n"/>
       <c r="R255" s="4" t="n"/>
       <c r="S255" s="4" t="n"/>
+      <c r="T255" s="4" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="4" t="n"/>
@@ -6076,6 +6343,7 @@
       <c r="Q256" s="4" t="n"/>
       <c r="R256" s="4" t="n"/>
       <c r="S256" s="4" t="n"/>
+      <c r="T256" s="4" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="4" t="n"/>
@@ -6097,6 +6365,7 @@
       <c r="Q257" s="4" t="n"/>
       <c r="R257" s="4" t="n"/>
       <c r="S257" s="4" t="n"/>
+      <c r="T257" s="4" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="4" t="n"/>
@@ -6118,6 +6387,7 @@
       <c r="Q258" s="4" t="n"/>
       <c r="R258" s="4" t="n"/>
       <c r="S258" s="4" t="n"/>
+      <c r="T258" s="4" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="4" t="n"/>
@@ -6139,6 +6409,7 @@
       <c r="Q259" s="4" t="n"/>
       <c r="R259" s="4" t="n"/>
       <c r="S259" s="4" t="n"/>
+      <c r="T259" s="4" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="4" t="n"/>
@@ -6160,6 +6431,7 @@
       <c r="Q260" s="4" t="n"/>
       <c r="R260" s="4" t="n"/>
       <c r="S260" s="4" t="n"/>
+      <c r="T260" s="4" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="4" t="n"/>
@@ -6181,6 +6453,7 @@
       <c r="Q261" s="4" t="n"/>
       <c r="R261" s="4" t="n"/>
       <c r="S261" s="4" t="n"/>
+      <c r="T261" s="4" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="4" t="n"/>
@@ -6202,6 +6475,7 @@
       <c r="Q262" s="4" t="n"/>
       <c r="R262" s="4" t="n"/>
       <c r="S262" s="4" t="n"/>
+      <c r="T262" s="4" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="4" t="n"/>
@@ -6223,6 +6497,7 @@
       <c r="Q263" s="4" t="n"/>
       <c r="R263" s="4" t="n"/>
       <c r="S263" s="4" t="n"/>
+      <c r="T263" s="4" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="n"/>
@@ -6244,6 +6519,7 @@
       <c r="Q264" s="4" t="n"/>
       <c r="R264" s="4" t="n"/>
       <c r="S264" s="4" t="n"/>
+      <c r="T264" s="4" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="4" t="n"/>
@@ -6265,6 +6541,7 @@
       <c r="Q265" s="4" t="n"/>
       <c r="R265" s="4" t="n"/>
       <c r="S265" s="4" t="n"/>
+      <c r="T265" s="4" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="n"/>
@@ -6286,6 +6563,7 @@
       <c r="Q266" s="4" t="n"/>
       <c r="R266" s="4" t="n"/>
       <c r="S266" s="4" t="n"/>
+      <c r="T266" s="4" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="n"/>
@@ -6307,6 +6585,7 @@
       <c r="Q267" s="4" t="n"/>
       <c r="R267" s="4" t="n"/>
       <c r="S267" s="4" t="n"/>
+      <c r="T267" s="4" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="4" t="n"/>
@@ -6328,6 +6607,7 @@
       <c r="Q268" s="4" t="n"/>
       <c r="R268" s="4" t="n"/>
       <c r="S268" s="4" t="n"/>
+      <c r="T268" s="4" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="4" t="n"/>
@@ -6349,6 +6629,7 @@
       <c r="Q269" s="4" t="n"/>
       <c r="R269" s="4" t="n"/>
       <c r="S269" s="4" t="n"/>
+      <c r="T269" s="4" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="4" t="n"/>
@@ -6370,6 +6651,7 @@
       <c r="Q270" s="4" t="n"/>
       <c r="R270" s="4" t="n"/>
       <c r="S270" s="4" t="n"/>
+      <c r="T270" s="4" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="4" t="n"/>
@@ -6391,6 +6673,7 @@
       <c r="Q271" s="4" t="n"/>
       <c r="R271" s="4" t="n"/>
       <c r="S271" s="4" t="n"/>
+      <c r="T271" s="4" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="4" t="n"/>
@@ -6412,6 +6695,7 @@
       <c r="Q272" s="4" t="n"/>
       <c r="R272" s="4" t="n"/>
       <c r="S272" s="4" t="n"/>
+      <c r="T272" s="4" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="n"/>
@@ -6433,6 +6717,7 @@
       <c r="Q273" s="4" t="n"/>
       <c r="R273" s="4" t="n"/>
       <c r="S273" s="4" t="n"/>
+      <c r="T273" s="4" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="4" t="n"/>
@@ -6454,6 +6739,7 @@
       <c r="Q274" s="4" t="n"/>
       <c r="R274" s="4" t="n"/>
       <c r="S274" s="4" t="n"/>
+      <c r="T274" s="4" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="4" t="n"/>
@@ -6475,6 +6761,7 @@
       <c r="Q275" s="4" t="n"/>
       <c r="R275" s="4" t="n"/>
       <c r="S275" s="4" t="n"/>
+      <c r="T275" s="4" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="n"/>
@@ -6496,6 +6783,7 @@
       <c r="Q276" s="4" t="n"/>
       <c r="R276" s="4" t="n"/>
       <c r="S276" s="4" t="n"/>
+      <c r="T276" s="4" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="4" t="n"/>
@@ -6517,6 +6805,7 @@
       <c r="Q277" s="4" t="n"/>
       <c r="R277" s="4" t="n"/>
       <c r="S277" s="4" t="n"/>
+      <c r="T277" s="4" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="4" t="n"/>
@@ -6538,6 +6827,7 @@
       <c r="Q278" s="4" t="n"/>
       <c r="R278" s="4" t="n"/>
       <c r="S278" s="4" t="n"/>
+      <c r="T278" s="4" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="4" t="n"/>
@@ -6559,6 +6849,7 @@
       <c r="Q279" s="4" t="n"/>
       <c r="R279" s="4" t="n"/>
       <c r="S279" s="4" t="n"/>
+      <c r="T279" s="4" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="4" t="n"/>
@@ -6580,6 +6871,7 @@
       <c r="Q280" s="4" t="n"/>
       <c r="R280" s="4" t="n"/>
       <c r="S280" s="4" t="n"/>
+      <c r="T280" s="4" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="4" t="n"/>
@@ -6601,6 +6893,7 @@
       <c r="Q281" s="4" t="n"/>
       <c r="R281" s="4" t="n"/>
       <c r="S281" s="4" t="n"/>
+      <c r="T281" s="4" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="4" t="n"/>
@@ -6622,6 +6915,7 @@
       <c r="Q282" s="4" t="n"/>
       <c r="R282" s="4" t="n"/>
       <c r="S282" s="4" t="n"/>
+      <c r="T282" s="4" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="4" t="n"/>
@@ -6643,6 +6937,7 @@
       <c r="Q283" s="4" t="n"/>
       <c r="R283" s="4" t="n"/>
       <c r="S283" s="4" t="n"/>
+      <c r="T283" s="4" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="4" t="n"/>
@@ -6664,6 +6959,7 @@
       <c r="Q284" s="4" t="n"/>
       <c r="R284" s="4" t="n"/>
       <c r="S284" s="4" t="n"/>
+      <c r="T284" s="4" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="4" t="n"/>
@@ -6685,6 +6981,7 @@
       <c r="Q285" s="4" t="n"/>
       <c r="R285" s="4" t="n"/>
       <c r="S285" s="4" t="n"/>
+      <c r="T285" s="4" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="4" t="n"/>
@@ -6706,6 +7003,7 @@
       <c r="Q286" s="4" t="n"/>
       <c r="R286" s="4" t="n"/>
       <c r="S286" s="4" t="n"/>
+      <c r="T286" s="4" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="4" t="n"/>
@@ -6727,6 +7025,7 @@
       <c r="Q287" s="4" t="n"/>
       <c r="R287" s="4" t="n"/>
       <c r="S287" s="4" t="n"/>
+      <c r="T287" s="4" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="4" t="n"/>
@@ -6748,6 +7047,7 @@
       <c r="Q288" s="4" t="n"/>
       <c r="R288" s="4" t="n"/>
       <c r="S288" s="4" t="n"/>
+      <c r="T288" s="4" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="4" t="n"/>
@@ -6769,6 +7069,7 @@
       <c r="Q289" s="4" t="n"/>
       <c r="R289" s="4" t="n"/>
       <c r="S289" s="4" t="n"/>
+      <c r="T289" s="4" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="4" t="n"/>
@@ -6790,6 +7091,7 @@
       <c r="Q290" s="4" t="n"/>
       <c r="R290" s="4" t="n"/>
       <c r="S290" s="4" t="n"/>
+      <c r="T290" s="4" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="4" t="n"/>
@@ -6811,6 +7113,7 @@
       <c r="Q291" s="4" t="n"/>
       <c r="R291" s="4" t="n"/>
       <c r="S291" s="4" t="n"/>
+      <c r="T291" s="4" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="4" t="n"/>
@@ -6832,6 +7135,7 @@
       <c r="Q292" s="4" t="n"/>
       <c r="R292" s="4" t="n"/>
       <c r="S292" s="4" t="n"/>
+      <c r="T292" s="4" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="4" t="n"/>
@@ -6853,6 +7157,7 @@
       <c r="Q293" s="4" t="n"/>
       <c r="R293" s="4" t="n"/>
       <c r="S293" s="4" t="n"/>
+      <c r="T293" s="4" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="4" t="n"/>
@@ -6874,6 +7179,7 @@
       <c r="Q294" s="4" t="n"/>
       <c r="R294" s="4" t="n"/>
       <c r="S294" s="4" t="n"/>
+      <c r="T294" s="4" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="4" t="n"/>
@@ -6895,6 +7201,7 @@
       <c r="Q295" s="4" t="n"/>
       <c r="R295" s="4" t="n"/>
       <c r="S295" s="4" t="n"/>
+      <c r="T295" s="4" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="4" t="n"/>
@@ -6916,6 +7223,7 @@
       <c r="Q296" s="4" t="n"/>
       <c r="R296" s="4" t="n"/>
       <c r="S296" s="4" t="n"/>
+      <c r="T296" s="4" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="4" t="n"/>
@@ -6937,6 +7245,7 @@
       <c r="Q297" s="4" t="n"/>
       <c r="R297" s="4" t="n"/>
       <c r="S297" s="4" t="n"/>
+      <c r="T297" s="4" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="n"/>
@@ -6958,6 +7267,7 @@
       <c r="Q298" s="4" t="n"/>
       <c r="R298" s="4" t="n"/>
       <c r="S298" s="4" t="n"/>
+      <c r="T298" s="4" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="4" t="n"/>
@@ -6979,6 +7289,7 @@
       <c r="Q299" s="4" t="n"/>
       <c r="R299" s="4" t="n"/>
       <c r="S299" s="4" t="n"/>
+      <c r="T299" s="4" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n"/>
@@ -7000,6 +7311,7 @@
       <c r="Q300" s="4" t="n"/>
       <c r="R300" s="4" t="n"/>
       <c r="S300" s="4" t="n"/>
+      <c r="T300" s="4" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="4" t="n"/>
@@ -7021,6 +7333,7 @@
       <c r="Q301" s="4" t="n"/>
       <c r="R301" s="4" t="n"/>
       <c r="S301" s="4" t="n"/>
+      <c r="T301" s="4" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="4" t="n"/>
@@ -7042,6 +7355,7 @@
       <c r="Q302" s="4" t="n"/>
       <c r="R302" s="4" t="n"/>
       <c r="S302" s="4" t="n"/>
+      <c r="T302" s="4" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="n"/>
@@ -7063,6 +7377,7 @@
       <c r="Q303" s="4" t="n"/>
       <c r="R303" s="4" t="n"/>
       <c r="S303" s="4" t="n"/>
+      <c r="T303" s="4" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="4" t="n"/>
@@ -7084,6 +7399,7 @@
       <c r="Q304" s="4" t="n"/>
       <c r="R304" s="4" t="n"/>
       <c r="S304" s="4" t="n"/>
+      <c r="T304" s="4" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="4" t="n"/>
@@ -7105,28 +7421,29 @@
       <c r="Q305" s="4" t="n"/>
       <c r="R305" s="4" t="n"/>
       <c r="S305" s="4" t="n"/>
+      <c r="T305" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A1:T1"/>
   </mergeCells>
   <dataValidations count="6">
-    <dataValidation sqref="B3:B305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: LAKI_LAKI, PEREMPUAN" type="list">
+    <dataValidation sqref="C3:C305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: LAKI_LAKI, PEREMPUAN" type="list">
       <formula1>"LAKI_LAKI,PEREMPUAN"</formula1>
     </dataValidation>
-    <dataValidation sqref="E3:E305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: ISLAM, KRISTEN, KATOLIK, HINDU, BUDDHA, KONGHUCU, LAINNYA" type="list">
+    <dataValidation sqref="F3:F305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: ISLAM, KRISTEN, KATOLIK, HINDU, BUDDHA, KONGHUCU, LAINNYA" type="list">
       <formula1>"ISLAM,KRISTEN,KATOLIK,HINDU,BUDDHA,KONGHUCU,LAINNYA"</formula1>
     </dataValidation>
-    <dataValidation sqref="F3:F305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: BELUM_KAWIN, KAWIN, CERAI_HIDUP, CERAI_MATI" type="list">
+    <dataValidation sqref="G3:G305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: BELUM_KAWIN, KAWIN, CERAI_HIDUP, CERAI_MATI" type="list">
       <formula1>"BELUM_KAWIN,KAWIN,CERAI_HIDUP,CERAI_MATI"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: TIDAK_SEKOLAH, SD, SMP, SMA, D3, S1, S2, S3" type="list">
+    <dataValidation sqref="H3:H305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: TIDAK_SEKOLAH, SD, SMP, SMA, D3, S1, S2, S3" type="list">
       <formula1>"TIDAK_SEKOLAH,SD,SMP,SMA,D3,S1,S2,S3"</formula1>
     </dataValidation>
-    <dataValidation sqref="I3:I305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: A, B, AB, O, TIDAK_TAHU" type="list">
+    <dataValidation sqref="J3:J305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: A, B, AB, O, TIDAK_TAHU" type="list">
       <formula1>"A,B,AB,O,TIDAK_TAHU"</formula1>
     </dataValidation>
-    <dataValidation sqref="J3:J305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: KEPALA_KELUARGA, ISTRI, ANAK, FAMILI_LAIN, LAINNYA" type="list">
+    <dataValidation sqref="K3:K305" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih salah satu: KEPALA_KELUARGA, ISTRI, ANAK, FAMILI_LAIN, LAINNYA" type="list">
       <formula1>"KEPALA_KELUARGA,ISTRI,ANAK,FAMILI_LAIN,LAINNYA"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7140,7 +7457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -7185,49 +7502,94 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>4. Tanggal Lahir: format yyyy-mm-dd (contoh 1990-01-01).</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5. Kolom berikut WAJIB pilih dari dropdown (klik sel, muncul panah di kanan):</t>
+          <t xml:space="preserve">   KODE WARGA — kolom paling penting:</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Jenis Kelamin, Agama, Status Perkawinan, Pendidikan Terakhir,</t>
+          <t xml:space="preserve">   - Wajib diisi, tidak boleh kosong, tidak boleh sama dengan warga lain.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Gol. Darah, Status dalam Keluarga.</t>
+          <t xml:space="preserve">   - Sekali diberikan, JANGAN PERNAH diubah. Kode inilah yang dipakai</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6. Kirim file LENGKAP berisi SELURUH warga, bukan tambahannya saja:</t>
+          <t xml:space="preserve">     sistem untuk mengenali orang yang sama pada pendataan berikutnya.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   impor menimpa seluruh data lama.</t>
+          <t xml:space="preserve">   - Warga baru mendapat kode berikutnya yang belum terpakai; kode milik</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     warga yang meninggal atau pindah JANGAN dipakai ulang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4. Tanggal Lahir: format yyyy-mm-dd (contoh 1990-01-01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>5. Kolom berikut WAJIB pilih dari dropdown (klik sel, muncul panah di kanan):</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Jenis Kelamin, Agama, Status Perkawinan, Pendidikan Terakhir,</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Gol. Darah, Status dalam Keluarga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>6. Kirim file LENGKAP berisi SELURUH warga, bukan tambahannya saja:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   impor menimpa seluruh data lama.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>7. Simpan sebagai .xlsx, kirim ke pengelola data untuk diimpor ke sistem.</t>
         </is>

</xml_diff>